<commit_message>
codex: compile stock and statistical balance aliases
Verification: 6 focused mapping/parser tests passed; canonical refresh promoted and reopened successfully; workbook error scan found no formula error tokens.
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0fcfe5e897c94e9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="Rb5b34152cee540fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R7cc1ff5b5c7048ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R2b3121930cdc4a74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R92ae984d2c934895"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R24420ba3b0c24893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="R7c16a4257cdf47bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="R04051ca78b834f29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="Rb77729cdc45648c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R81c7e2016ac24af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R165ebea1310044af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd5a04c2b4a784b9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="Raf517561891449c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R5f4ce45fe51d4f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R15a9de2067344e8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R5add99920203428c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Rfe7ad548d9c949e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="R5f9279f3c8f74b3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Rc83eeef31c014233"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="Rd4c7fe93fc0849c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R2712722cdb164887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R211d1f1de7b74de8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16037,87 +16037,87 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="28" t="str">
-        <x:v>Charcoal processing/Charcoal processing</x:v>
+        <x:v>CHP plants/Processes/Coal CHP</x:v>
       </x:c>
       <x:c r="B16" s="28" t="str">
-        <x:v>09.11 Charcoal processing</x:v>
+        <x:v>09.02.02.01 Coal CHP</x:v>
       </x:c>
       <x:c r="C16" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="28" t="str">
-        <x:v>Chemical heat for electricity production/Chemical heat for electricity production</x:v>
+        <x:v>CHP plants/Processes/Gas CHP</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>09.05 Chemical heat for electricity production</x:v>
+        <x:v>09.01.02.02 Gas CHP</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="28" t="str">
-        <x:v>Coal transformation</x:v>
+        <x:v>CHP plants/Processes/Gas CHP</x:v>
       </x:c>
       <x:c r="B18" s="28" t="str">
-        <x:v>09.08 Coal transformation</x:v>
+        <x:v>09.02.02.02 Gas CHP</x:v>
       </x:c>
       <x:c r="C18" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="28" t="str">
-        <x:v>Coke ovens/Coke ovens</x:v>
+        <x:v>CHP plants/Processes/Others CHP</x:v>
       </x:c>
       <x:c r="B19" s="28" t="str">
-        <x:v>09.08.01 Coke ovens (including own use)</x:v>
+        <x:v>09.01.02.03 Others CHP</x:v>
       </x:c>
       <x:c r="C19" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="28" t="str">
-        <x:v>Demand\All demand aggregated\International transport</x:v>
+        <x:v>CHP plants/Processes/Others CHP</x:v>
       </x:c>
       <x:c r="B20" s="28" t="str">
-        <x:v>04-05 International transport (bunkers)</x:v>
+        <x:v>09.02.02.03 Others CHP</x:v>
       </x:c>
       <x:c r="C20" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="28" t="str">
-        <x:v>Demand\All demand aggregated\Other sector</x:v>
+        <x:v>CHP plants/Processes/Petroleum products CHP</x:v>
       </x:c>
       <x:c r="B21" s="28" t="str">
-        <x:v>16.03-16.05 Other sector (all demand aggregate)</x:v>
+        <x:v>09.01.02.04 Petroleum products CHP</x:v>
       </x:c>
       <x:c r="C21" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="28" t="str">
-        <x:v>Demand\All demand aggregated\Road</x:v>
+        <x:v>CHP plants/Processes/Petroleum products CHP</x:v>
       </x:c>
       <x:c r="B22" s="28" t="str">
-        <x:v>15.02 Road</x:v>
+        <x:v>09.02.02.04 Petroleum products CHP</x:v>
       </x:c>
       <x:c r="C22" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="28" t="str">
-        <x:v>Demand\All demand aggregated\Transport non road</x:v>
+        <x:v>Charcoal processing/Charcoal processing</x:v>
       </x:c>
       <x:c r="B23" s="28" t="str">
-        <x:v>15.01,15.03-15.06 Transport non-road</x:v>
+        <x:v>09.11 Charcoal processing</x:v>
       </x:c>
       <x:c r="C23" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16125,10 +16125,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="28" t="str">
-        <x:v>Electric boilers/Electric boilers</x:v>
+        <x:v>Chemical heat for electricity production/Chemical heat for electricity production</x:v>
       </x:c>
       <x:c r="B24" s="28" t="str">
-        <x:v>09.04 Electric boilers</x:v>
+        <x:v>09.05 Chemical heat for electricity production</x:v>
       </x:c>
       <x:c r="C24" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16136,10 +16136,10 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="28" t="str">
-        <x:v>Electricity Generation</x:v>
+        <x:v>Coal transformation</x:v>
       </x:c>
       <x:c r="B25" s="28" t="str">
-        <x:v>09.01.01,09.02.01 Electricity plants</x:v>
+        <x:v>09.08 Coal transformation</x:v>
       </x:c>
       <x:c r="C25" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16147,10 +16147,10 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="28" t="str">
-        <x:v>Electricity interim/Electricity interim</x:v>
+        <x:v>Coke ovens/Coke ovens</x:v>
       </x:c>
       <x:c r="B26" s="28" t="str">
-        <x:v>09.01.01,09.02.01 Electricity plants</x:v>
+        <x:v>09.08.01 Coke ovens (including own use)</x:v>
       </x:c>
       <x:c r="C26" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16158,10 +16158,10 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="28" t="str">
-        <x:v>Exports</x:v>
+        <x:v>Demand\All demand aggregated\International transport</x:v>
       </x:c>
       <x:c r="B27" s="28" t="str">
-        <x:v>03 Exports</x:v>
+        <x:v>04-05 International transport (bunkers)</x:v>
       </x:c>
       <x:c r="C27" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16169,10 +16169,10 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="28" t="str">
-        <x:v>Gas processing plants</x:v>
+        <x:v>Demand\All demand aggregated\Other sector</x:v>
       </x:c>
       <x:c r="B28" s="28" t="str">
-        <x:v>09.06 Gas processing plants</x:v>
+        <x:v>16.03-16.05 Other sector (all demand aggregate)</x:v>
       </x:c>
       <x:c r="C28" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16180,10 +16180,10 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="28" t="str">
-        <x:v>Gas to liquids plants/Gas to liquids plants</x:v>
+        <x:v>Demand\All demand aggregated\Road</x:v>
       </x:c>
       <x:c r="B29" s="28" t="str">
-        <x:v>09.06.04 Gas-to-liquids plants</x:v>
+        <x:v>15.02 Road</x:v>
       </x:c>
       <x:c r="C29" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16191,10 +16191,10 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="28" t="str">
-        <x:v>Gas works plants/Gas works plants</x:v>
+        <x:v>Demand\All demand aggregated\Transport non road</x:v>
       </x:c>
       <x:c r="B30" s="28" t="str">
-        <x:v>09.06.01 Gas works plants (including own use)</x:v>
+        <x:v>15.01,15.03-15.06 Transport non-road</x:v>
       </x:c>
       <x:c r="C30" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16202,10 +16202,10 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="28" t="str">
-        <x:v>Heat plant interim/Heat plant interim</x:v>
+        <x:v>Electric boilers/Electric boilers</x:v>
       </x:c>
       <x:c r="B31" s="28" t="str">
-        <x:v>09.01.03,09.02.03 Heat plants</x:v>
+        <x:v>09.04 Electric boilers</x:v>
       </x:c>
       <x:c r="C31" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16213,10 +16213,10 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="28" t="str">
-        <x:v>Heat plants</x:v>
+        <x:v>Electricity Generation</x:v>
       </x:c>
       <x:c r="B32" s="28" t="str">
-        <x:v>09.01.03,09.02.03 Heat plants</x:v>
+        <x:v>09.01.01,09.02.01 Electricity plants</x:v>
       </x:c>
       <x:c r="C32" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16224,10 +16224,10 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="28" t="str">
-        <x:v>Hydrogen transformation</x:v>
+        <x:v>Electricity interim/Electricity interim</x:v>
       </x:c>
       <x:c r="B33" s="28" t="str">
-        <x:v>09.13 Hydrogen transformation</x:v>
+        <x:v>09.01.01,09.02.01 Electricity plants</x:v>
       </x:c>
       <x:c r="C33" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16235,10 +16235,10 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="28" t="str">
-        <x:v>Hydrogen transformation/Electrolysers</x:v>
+        <x:v>Exports</x:v>
       </x:c>
       <x:c r="B34" s="28" t="str">
-        <x:v>09.13.01 Electrolysers</x:v>
+        <x:v>03 Exports</x:v>
       </x:c>
       <x:c r="C34" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16246,142 +16246,142 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="28" t="str">
-        <x:v>Hydrogen transformation/SMR with CCS</x:v>
+        <x:v>Freight road</x:v>
       </x:c>
       <x:c r="B35" s="28" t="str">
-        <x:v>09.13.03 SMR w CCS</x:v>
+        <x:v>15.02.01 Freight road</x:v>
       </x:c>
       <x:c r="C35" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="28" t="str">
-        <x:v>Imports</x:v>
+        <x:v>Freight road/LCVs</x:v>
       </x:c>
       <x:c r="B36" s="28" t="str">
-        <x:v>02 Imports</x:v>
+        <x:v>15.02.01.01 LCVs</x:v>
       </x:c>
       <x:c r="C36" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="28" t="str">
-        <x:v>Industry</x:v>
+        <x:v>Freight road/LCVs/BEV</x:v>
       </x:c>
       <x:c r="B37" s="28" t="str">
-        <x:v>14 Industry sector</x:v>
+        <x:v>15.02.01.01.01 BEV</x:v>
       </x:c>
       <x:c r="C37" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="28" t="str">
-        <x:v>Industry/Construction</x:v>
+        <x:v>Freight road/LCVs/ICE</x:v>
       </x:c>
       <x:c r="B38" s="28" t="str">
-        <x:v>14.02 Construction</x:v>
+        <x:v>15.02.01.01.02 ICE</x:v>
       </x:c>
       <x:c r="C38" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="28" t="str">
-        <x:v>Industry/Manufacturing</x:v>
+        <x:v>Freight road/LCVs/PHEV</x:v>
       </x:c>
       <x:c r="B39" s="28" t="str">
-        <x:v>14.03 Manufacturing</x:v>
+        <x:v>15.02.01.01.03 PHEV</x:v>
       </x:c>
       <x:c r="C39" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="28" t="str">
-        <x:v>Industry/Manufacturing/Chemical</x:v>
+        <x:v>Freight road/Trucks</x:v>
       </x:c>
       <x:c r="B40" s="28" t="str">
-        <x:v>14.03.02 Chemical (incl. petrochemical)</x:v>
+        <x:v>15.02.01.02 Trucks</x:v>
       </x:c>
       <x:c r="C40" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="28" t="str">
-        <x:v>Industry/Manufacturing/Food beverages and tobacco</x:v>
+        <x:v>Freight road/Trucks/BEV heavy</x:v>
       </x:c>
       <x:c r="B41" s="28" t="str">
-        <x:v>14.03.07 Food, beverages and tobacco</x:v>
+        <x:v>15.02.01.02.01 BEV heavy</x:v>
       </x:c>
       <x:c r="C41" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="28" t="str">
-        <x:v>Industry/Manufacturing/Iron and steel</x:v>
+        <x:v>Freight road/Trucks/BEV medium</x:v>
       </x:c>
       <x:c r="B42" s="28" t="str">
-        <x:v>14.03.01 Iron and steel</x:v>
+        <x:v>15.02.01.02.02 BEV medium</x:v>
       </x:c>
       <x:c r="C42" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="28" t="str">
-        <x:v>Industry/Manufacturing/Machinery</x:v>
+        <x:v>Freight road/Trucks/FCEV heavy</x:v>
       </x:c>
       <x:c r="B43" s="28" t="str">
-        <x:v>14.03.06 Machinery</x:v>
+        <x:v>15.02.01.02.03 FCEV heavy</x:v>
       </x:c>
       <x:c r="C43" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="28" t="str">
-        <x:v>Industry/Manufacturing/Non ferrous metals</x:v>
+        <x:v>Freight road/Trucks/FCEV medium</x:v>
       </x:c>
       <x:c r="B44" s="28" t="str">
-        <x:v>14.03.03 Non ferrous metals</x:v>
+        <x:v>15.02.01.02.04 FCEV medium</x:v>
       </x:c>
       <x:c r="C44" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="28" t="str">
-        <x:v>Industry/Manufacturing/Non metallic mineral products</x:v>
+        <x:v>Freight road/Trucks/ICE heavy</x:v>
       </x:c>
       <x:c r="B45" s="28" t="str">
-        <x:v>14.03.04 Non-metallic mineral products</x:v>
+        <x:v>15.02.01.02.05 ICE heavy</x:v>
       </x:c>
       <x:c r="C45" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="28" t="str">
-        <x:v>Industry/Manufacturing/Non specified industry</x:v>
+        <x:v>Freight road/Trucks/ICE medium</x:v>
       </x:c>
       <x:c r="B46" s="28" t="str">
-        <x:v>14.03.11 Non-specified industry</x:v>
+        <x:v>15.02.01.02.06 ICE medium</x:v>
       </x:c>
       <x:c r="C46" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="28" t="str">
-        <x:v>Industry/Manufacturing/Pulp paper and printing</x:v>
+        <x:v>Gas processing plants</x:v>
       </x:c>
       <x:c r="B47" s="28" t="str">
-        <x:v>14.03.08 Pulp, paper and printing</x:v>
+        <x:v>09.06 Gas processing plants</x:v>
       </x:c>
       <x:c r="C47" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16389,10 +16389,10 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="28" t="str">
-        <x:v>Industry/Manufacturing/Textiles and leather</x:v>
+        <x:v>Gas to liquids plants/Gas to liquids plants</x:v>
       </x:c>
       <x:c r="B48" s="28" t="str">
-        <x:v>14.03.10 Textiles and leather</x:v>
+        <x:v>09.06.04 Gas-to-liquids plants</x:v>
       </x:c>
       <x:c r="C48" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16400,10 +16400,10 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="28" t="str">
-        <x:v>Industry/Manufacturing/Transportation equipment</x:v>
+        <x:v>Gas works plants/Gas works plants</x:v>
       </x:c>
       <x:c r="B49" s="28" t="str">
-        <x:v>14.03.05 Transportation equipment</x:v>
+        <x:v>09.06.01 Gas works plants (including own use)</x:v>
       </x:c>
       <x:c r="C49" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16411,10 +16411,10 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="28" t="str">
-        <x:v>Industry/Manufacturing/Wood and wood products</x:v>
+        <x:v>Heat plant interim/Heat plant interim</x:v>
       </x:c>
       <x:c r="B50" s="28" t="str">
-        <x:v>14.03.09 Wood and wood products</x:v>
+        <x:v>09.01.03,09.02.03 Heat plants</x:v>
       </x:c>
       <x:c r="C50" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16422,10 +16422,10 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="28" t="str">
-        <x:v>Industry/Mining and quarrying</x:v>
+        <x:v>Heat plants</x:v>
       </x:c>
       <x:c r="B51" s="28" t="str">
-        <x:v>14.01 Mining and quarrying</x:v>
+        <x:v>09.01.03,09.02.03 Heat plants</x:v>
       </x:c>
       <x:c r="C51" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16433,98 +16433,98 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="28" t="str">
-        <x:v>International transport</x:v>
+        <x:v>Heat plants/Processes/Coal HP</x:v>
       </x:c>
       <x:c r="B52" s="28" t="str">
-        <x:v>04-05 International transport (bunkers)</x:v>
+        <x:v>09.01.03.01 Coal HP</x:v>
       </x:c>
       <x:c r="C52" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="28" t="str">
-        <x:v>LNG regasification/Regasification</x:v>
+        <x:v>Heat plants/Processes/Coal HP</x:v>
       </x:c>
       <x:c r="B53" s="28" t="str">
-        <x:v>09.06.02.01 Liquefaction</x:v>
+        <x:v>09.02.03.01 Coal HP</x:v>
       </x:c>
       <x:c r="C53" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="28" t="str">
-        <x:v>LNG regasification/Regasification</x:v>
+        <x:v>Heat plants/Processes/Gas HP</x:v>
       </x:c>
       <x:c r="B54" s="28" t="str">
-        <x:v>09.06.02.02 Regasification</x:v>
+        <x:v>09.01.03.02 Gas HP</x:v>
       </x:c>
       <x:c r="C54" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="28" t="str">
-        <x:v>Liquefaction coal to oil/Liquefaction coal to oil</x:v>
+        <x:v>Heat plants/Processes/Gas HP</x:v>
       </x:c>
       <x:c r="B55" s="28" t="str">
-        <x:v>09.08.05 Liquefaction (coal to oil)</x:v>
+        <x:v>09.02.03.02 Gas HP</x:v>
       </x:c>
       <x:c r="C55" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="28" t="str">
-        <x:v>Liquefaction/regasification plants</x:v>
+        <x:v>Heat plants/Processes/Others HP</x:v>
       </x:c>
       <x:c r="B56" s="28" t="str">
-        <x:v>09.06.02 Liquefaction/regasification plants</x:v>
+        <x:v>09.01.03.03 Others HP</x:v>
       </x:c>
       <x:c r="C56" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="28" t="str">
-        <x:v>NG Liquefaction/Liquefaction</x:v>
+        <x:v>Heat plants/Processes/Others HP</x:v>
       </x:c>
       <x:c r="B57" s="28" t="str">
-        <x:v>09.06.02.01 Liquefaction</x:v>
+        <x:v>09.02.03.03 Others HP</x:v>
       </x:c>
       <x:c r="C57" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="28" t="str">
-        <x:v>NG Liquefaction/NG Liquefaction</x:v>
+        <x:v>Heat plants/Processes/Petroleum products HP</x:v>
       </x:c>
       <x:c r="B58" s="28" t="str">
-        <x:v>09.06.02.01 Liquefaction</x:v>
+        <x:v>09.01.03.04 Petroleum products HP</x:v>
       </x:c>
       <x:c r="C58" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="28" t="str">
-        <x:v>Natural gas blending plants/Natural gas blending plants</x:v>
+        <x:v>Heat plants/Processes/Petroleum products HP</x:v>
       </x:c>
       <x:c r="B59" s="28" t="str">
-        <x:v>09.06.03 Natural gas blending plants</x:v>
+        <x:v>09.02.03.04 Petroleum products HP</x:v>
       </x:c>
       <x:c r="C59" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="28" t="str">
-        <x:v>Non specified transformation/Non specified transformation</x:v>
+        <x:v>Hydrogen transformation</x:v>
       </x:c>
       <x:c r="B60" s="28" t="str">
-        <x:v>09.12 Non-specified transformation</x:v>
+        <x:v>09.13 Hydrogen transformation</x:v>
       </x:c>
       <x:c r="C60" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16532,10 +16532,10 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="28" t="str">
-        <x:v>Non-energy use</x:v>
+        <x:v>Hydrogen transformation/Electrolysers</x:v>
       </x:c>
       <x:c r="B61" s="28" t="str">
-        <x:v>17 Non-energy use</x:v>
+        <x:v>09.13.01 Electrolysers</x:v>
       </x:c>
       <x:c r="C61" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16543,21 +16543,21 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="28" t="str">
-        <x:v>Oil Refining/Oil Refining</x:v>
+        <x:v>Hydrogen transformation/Processes/SMR with CCS</x:v>
       </x:c>
       <x:c r="B62" s="28" t="str">
-        <x:v>09.07 Oil refineries</x:v>
+        <x:v>09.13.02 SMR with CCS</x:v>
       </x:c>
       <x:c r="C62" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="28" t="str">
-        <x:v>Other loss and own use/Coal mines</x:v>
+        <x:v>Hydrogen transformation/SMR with CCS</x:v>
       </x:c>
       <x:c r="B63" s="28" t="str">
-        <x:v>10.01.06 Coal mines</x:v>
+        <x:v>09.13.03 SMR w CCS</x:v>
       </x:c>
       <x:c r="C63" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16565,10 +16565,10 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="28" t="str">
-        <x:v>Other loss and own use/Electricity CHP and heat plants</x:v>
+        <x:v>Imports</x:v>
       </x:c>
       <x:c r="B64" s="28" t="str">
-        <x:v>10.01.01 Electricity, CHP and heat plants</x:v>
+        <x:v>02 Imports</x:v>
       </x:c>
       <x:c r="C64" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16576,10 +16576,10 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="28" t="str">
-        <x:v>Other loss and own use/Liquefaction and regasification plants</x:v>
+        <x:v>Industry</x:v>
       </x:c>
       <x:c r="B65" s="28" t="str">
-        <x:v>10.01.03 Liquefaction/regasification plants</x:v>
+        <x:v>14 Industry sector</x:v>
       </x:c>
       <x:c r="C65" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16587,10 +16587,10 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="28" t="str">
-        <x:v>Other loss and own use/Non specified own uses</x:v>
+        <x:v>Industry/Construction</x:v>
       </x:c>
       <x:c r="B66" s="28" t="str">
-        <x:v>10.01.17 Non-specified own uses</x:v>
+        <x:v>14.02 Construction</x:v>
       </x:c>
       <x:c r="C66" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16598,10 +16598,10 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="28" t="str">
-        <x:v>Other loss and own use/Oil and gas extraction</x:v>
+        <x:v>Industry/Manufacturing</x:v>
       </x:c>
       <x:c r="B67" s="28" t="str">
-        <x:v>10.01.12 Oil and gas extraction</x:v>
+        <x:v>14.03 Manufacturing</x:v>
       </x:c>
       <x:c r="C67" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16609,10 +16609,10 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="28" t="str">
-        <x:v>Other loss and own use/Oil refineries</x:v>
+        <x:v>Industry/Manufacturing/Chemical</x:v>
       </x:c>
       <x:c r="B68" s="28" t="str">
-        <x:v>10.01.11 Oil refineries</x:v>
+        <x:v>14.03.02 Chemical (incl. petrochemical)</x:v>
       </x:c>
       <x:c r="C68" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16620,10 +16620,10 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="28" t="str">
-        <x:v>Other loss and own use/Pump storage plants</x:v>
+        <x:v>Industry/Manufacturing/Food beverages and tobacco</x:v>
       </x:c>
       <x:c r="B69" s="28" t="str">
-        <x:v>10.01.13 Pump storage plants</x:v>
+        <x:v>14.03.07 Food, beverages and tobacco</x:v>
       </x:c>
       <x:c r="C69" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16631,10 +16631,10 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="28" t="str">
-        <x:v>Other loss and own use/Transmission and distribution loss</x:v>
+        <x:v>Industry/Manufacturing/Iron and steel</x:v>
       </x:c>
       <x:c r="B70" s="28" t="str">
-        <x:v>10.02 Transmission and distribution losses</x:v>
+        <x:v>14.03.01 Iron and steel</x:v>
       </x:c>
       <x:c r="C70" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16642,43 +16642,43 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="28" t="str">
-        <x:v>Other sector</x:v>
+        <x:v>Industry/Manufacturing/Iron and steel/Blast Furnace Basic Oxygen Furnace</x:v>
       </x:c>
       <x:c r="B71" s="28" t="str">
-        <x:v>16.03-16.05 Other sector (all demand aggregate)</x:v>
+        <x:v>14.03.01.01 Blast Furnace Basic Oxygen Furnace</x:v>
       </x:c>
       <x:c r="C71" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="28" t="str">
-        <x:v>Other sector/Agriculture</x:v>
+        <x:v>Industry/Manufacturing/Iron and steel/Direct Reduced Iron Electric Arc Furnace</x:v>
       </x:c>
       <x:c r="B72" s="28" t="str">
-        <x:v>16.03 Agriculture</x:v>
+        <x:v>14.03.01.02 Direct Reduced Iron Electric Arc Furnace</x:v>
       </x:c>
       <x:c r="C72" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="28" t="str">
-        <x:v>Other sector/Fishing</x:v>
+        <x:v>Industry/Manufacturing/Iron and steel/Scrap Electric Arc Furnace</x:v>
       </x:c>
       <x:c r="B73" s="28" t="str">
-        <x:v>16.04 Fishing</x:v>
+        <x:v>14.03.01.03 Scrap Electric Arc Furnace</x:v>
       </x:c>
       <x:c r="C73" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="28" t="str">
-        <x:v>Other sector/Non specified others</x:v>
+        <x:v>Industry/Manufacturing/Machinery</x:v>
       </x:c>
       <x:c r="B74" s="28" t="str">
-        <x:v>16.05 Non-specified others</x:v>
+        <x:v>14.03.06 Machinery</x:v>
       </x:c>
       <x:c r="C74" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16686,10 +16686,10 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="28" t="str">
-        <x:v>Patent fuel plants/Patent fuel plants</x:v>
+        <x:v>Industry/Manufacturing/Non ferrous metals</x:v>
       </x:c>
       <x:c r="B75" s="28" t="str">
-        <x:v>09.08.03 Patent fuel plants</x:v>
+        <x:v>14.03.03 Non ferrous metals</x:v>
       </x:c>
       <x:c r="C75" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16697,10 +16697,10 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="28" t="str">
-        <x:v>Petrochemical industry/Petrochemical industry</x:v>
+        <x:v>Industry/Manufacturing/Non metallic mineral products</x:v>
       </x:c>
       <x:c r="B76" s="28" t="str">
-        <x:v>09.09 Petrochemical industry</x:v>
+        <x:v>14.03.04 Non-metallic mineral products</x:v>
       </x:c>
       <x:c r="C76" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16708,10 +16708,10 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="28" t="str">
-        <x:v>Power</x:v>
+        <x:v>Industry/Manufacturing/Non specified industry</x:v>
       </x:c>
       <x:c r="B77" s="28" t="str">
-        <x:v>09.01-09.02 Power sector</x:v>
+        <x:v>14.03.11 Non-specified industry</x:v>
       </x:c>
       <x:c r="C77" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16719,10 +16719,10 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="28" t="str">
-        <x:v>Production</x:v>
+        <x:v>Industry/Manufacturing/Pulp paper and printing</x:v>
       </x:c>
       <x:c r="B78" s="28" t="str">
-        <x:v>01 Production</x:v>
+        <x:v>14.03.08 Pulp, paper and printing</x:v>
       </x:c>
       <x:c r="C78" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16730,10 +16730,10 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="28" t="str">
-        <x:v>Road</x:v>
+        <x:v>Industry/Manufacturing/Textiles and leather</x:v>
       </x:c>
       <x:c r="B79" s="28" t="str">
-        <x:v>15.02 Road</x:v>
+        <x:v>14.03.10 Textiles and leather</x:v>
       </x:c>
       <x:c r="C79" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16741,10 +16741,10 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="28" t="str">
-        <x:v>Total Primary Supply</x:v>
+        <x:v>Industry/Manufacturing/Transportation equipment</x:v>
       </x:c>
       <x:c r="B80" s="28" t="str">
-        <x:v>07 Total primary energy supply</x:v>
+        <x:v>14.03.05 Transportation equipment</x:v>
       </x:c>
       <x:c r="C80" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16752,10 +16752,10 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="28" t="str">
-        <x:v>Total final consumption</x:v>
+        <x:v>Industry/Manufacturing/Wood and wood products</x:v>
       </x:c>
       <x:c r="B81" s="28" t="str">
-        <x:v>12 Total final consumption</x:v>
+        <x:v>14.03.09 Wood and wood products</x:v>
       </x:c>
       <x:c r="C81" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16763,10 +16763,10 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="28" t="str">
-        <x:v>Total final energy consumption</x:v>
+        <x:v>Industry/Mining and quarrying</x:v>
       </x:c>
       <x:c r="B82" s="28" t="str">
-        <x:v>13 Total final energy consumption</x:v>
+        <x:v>14.01 Mining and quarrying</x:v>
       </x:c>
       <x:c r="C82" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16774,10 +16774,10 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="28" t="str">
-        <x:v>Total transformation - no transfers</x:v>
+        <x:v>International transport</x:v>
       </x:c>
       <x:c r="B83" s="28" t="str">
-        <x:v>09 Total transformation sector</x:v>
+        <x:v>04-05 International transport (bunkers)</x:v>
       </x:c>
       <x:c r="C83" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16785,10 +16785,10 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="28" t="str">
-        <x:v>Transfers</x:v>
+        <x:v>LNG regasification/Regasification</x:v>
       </x:c>
       <x:c r="B84" s="28" t="str">
-        <x:v>08 Transfers</x:v>
+        <x:v>09.06.02.01 Liquefaction</x:v>
       </x:c>
       <x:c r="C84" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16796,10 +16796,10 @@
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="28" t="str">
-        <x:v>Transmission and Distribution</x:v>
+        <x:v>LNG regasification/Regasification</x:v>
       </x:c>
       <x:c r="B85" s="28" t="str">
-        <x:v>10.02 Transmission and distribution losses</x:v>
+        <x:v>09.06.02.02 Regasification</x:v>
       </x:c>
       <x:c r="C85" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16807,10 +16807,10 @@
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="28" t="str">
-        <x:v>Transport</x:v>
+        <x:v>Liquefaction coal to oil/Liquefaction coal to oil</x:v>
       </x:c>
       <x:c r="B86" s="28" t="str">
-        <x:v>15 Transport sector</x:v>
+        <x:v>09.08.05 Liquefaction (coal to oil)</x:v>
       </x:c>
       <x:c r="C86" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16818,10 +16818,10 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="28" t="str">
-        <x:v>Transport non road</x:v>
+        <x:v>Liquefaction/regasification plants</x:v>
       </x:c>
       <x:c r="B87" s="28" t="str">
-        <x:v>15.01,15.03-15.06 Transport non-road</x:v>
+        <x:v>09.06.02 Liquefaction/regasification plants</x:v>
       </x:c>
       <x:c r="C87" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16829,10 +16829,10 @@
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="28" t="str">
-        <x:v>Transport non road/Freight non road/Air</x:v>
+        <x:v>NG Liquefaction/Liquefaction</x:v>
       </x:c>
       <x:c r="B88" s="28" t="str">
-        <x:v>15.01 Domestic air transport</x:v>
+        <x:v>09.06.02.01 Liquefaction</x:v>
       </x:c>
       <x:c r="C88" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16840,10 +16840,10 @@
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="28" t="str">
-        <x:v>Transport non road/Freight non road/Rail</x:v>
+        <x:v>NG Liquefaction/NG Liquefaction</x:v>
       </x:c>
       <x:c r="B89" s="28" t="str">
-        <x:v>15.03 Rail</x:v>
+        <x:v>09.06.02.01 Liquefaction</x:v>
       </x:c>
       <x:c r="C89" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16851,10 +16851,10 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="28" t="str">
-        <x:v>Transport non road/Freight non road/Shipping</x:v>
+        <x:v>Natural gas blending plants/Natural gas blending plants</x:v>
       </x:c>
       <x:c r="B90" s="28" t="str">
-        <x:v>15.04 Domestic navigation</x:v>
+        <x:v>09.06.03 Natural gas blending plants</x:v>
       </x:c>
       <x:c r="C90" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16862,10 +16862,10 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="28" t="str">
-        <x:v>Transport non road/International transport/Air</x:v>
+        <x:v>Non specified transformation/Non specified transformation</x:v>
       </x:c>
       <x:c r="B91" s="28" t="str">
-        <x:v>05 International aviation bunkers</x:v>
+        <x:v>09.12 Non-specified transformation</x:v>
       </x:c>
       <x:c r="C91" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16873,10 +16873,10 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="28" t="str">
-        <x:v>Transport non road/International transport/Shipping</x:v>
+        <x:v>Non-energy use</x:v>
       </x:c>
       <x:c r="B92" s="28" t="str">
-        <x:v>04 International marine bunkers</x:v>
+        <x:v>17 Non-energy use</x:v>
       </x:c>
       <x:c r="C92" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16884,10 +16884,10 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="28" t="str">
-        <x:v>Transport non road/Nonspecified transport</x:v>
+        <x:v>Oil Refining/Oil Refining</x:v>
       </x:c>
       <x:c r="B93" s="28" t="str">
-        <x:v>15.02 Road</x:v>
+        <x:v>09.07 Oil refineries</x:v>
       </x:c>
       <x:c r="C93" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16895,10 +16895,10 @@
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="28" t="str">
-        <x:v>Transport non road/Nonspecified transport</x:v>
+        <x:v>Other loss and own use/Coal mines</x:v>
       </x:c>
       <x:c r="B94" s="28" t="str">
-        <x:v>15.03 Rail</x:v>
+        <x:v>10.01.06 Coal mines</x:v>
       </x:c>
       <x:c r="C94" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16906,10 +16906,10 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="28" t="str">
-        <x:v>Transport non road/Nonspecified transport</x:v>
+        <x:v>Other loss and own use/Electricity CHP and heat plants</x:v>
       </x:c>
       <x:c r="B95" s="28" t="str">
-        <x:v>15.06 Non-specified transport</x:v>
+        <x:v>10.01.01 Electricity, CHP and heat plants</x:v>
       </x:c>
       <x:c r="C95" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16917,10 +16917,10 @@
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="28" t="str">
-        <x:v>Transport non road/Passenger non road/Air</x:v>
+        <x:v>Other loss and own use/Liquefaction and regasification plants</x:v>
       </x:c>
       <x:c r="B96" s="28" t="str">
-        <x:v>15.01 Domestic air transport</x:v>
+        <x:v>10.01.03 Liquefaction/regasification plants</x:v>
       </x:c>
       <x:c r="C96" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16928,10 +16928,10 @@
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="28" t="str">
-        <x:v>Transport non road/Passenger non road/Rail</x:v>
+        <x:v>Other loss and own use/Non specified own uses</x:v>
       </x:c>
       <x:c r="B97" s="28" t="str">
-        <x:v>15.03 Rail</x:v>
+        <x:v>10.01.17 Non-specified own uses</x:v>
       </x:c>
       <x:c r="C97" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -16939,29 +16939,656 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="28" t="str">
+        <x:v>Other loss and own use/Oil and gas extraction</x:v>
+      </x:c>
+      <x:c r="B98" s="28" t="str">
+        <x:v>10.01.12 Oil and gas extraction</x:v>
+      </x:c>
+      <x:c r="C98" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="28" t="str">
+        <x:v>Other loss and own use/Oil refineries</x:v>
+      </x:c>
+      <x:c r="B99" s="28" t="str">
+        <x:v>10.01.11 Oil refineries</x:v>
+      </x:c>
+      <x:c r="C99" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="28" t="str">
+        <x:v>Other loss and own use/Pump storage plants</x:v>
+      </x:c>
+      <x:c r="B100" s="28" t="str">
+        <x:v>10.01.13 Pump storage plants</x:v>
+      </x:c>
+      <x:c r="C100" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="28" t="str">
+        <x:v>Other loss and own use/Transmission and distribution loss</x:v>
+      </x:c>
+      <x:c r="B101" s="28" t="str">
+        <x:v>10.02 Transmission and distribution losses</x:v>
+      </x:c>
+      <x:c r="C101" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="28" t="str">
+        <x:v>Other sector</x:v>
+      </x:c>
+      <x:c r="B102" s="28" t="str">
+        <x:v>16.03-16.05 Other sector (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="C102" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="28" t="str">
+        <x:v>Other sector/Agriculture</x:v>
+      </x:c>
+      <x:c r="B103" s="28" t="str">
+        <x:v>16.03 Agriculture</x:v>
+      </x:c>
+      <x:c r="C103" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="28" t="str">
+        <x:v>Other sector/Fishing</x:v>
+      </x:c>
+      <x:c r="B104" s="28" t="str">
+        <x:v>16.04 Fishing</x:v>
+      </x:c>
+      <x:c r="C104" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="28" t="str">
+        <x:v>Other sector/Non specified others</x:v>
+      </x:c>
+      <x:c r="B105" s="28" t="str">
+        <x:v>16.05 Non-specified others</x:v>
+      </x:c>
+      <x:c r="C105" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="28" t="str">
+        <x:v>Passenger road</x:v>
+      </x:c>
+      <x:c r="B106" s="28" t="str">
+        <x:v>15.02.02 Passenger road</x:v>
+      </x:c>
+      <x:c r="C106" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="28" t="str">
+        <x:v>Passenger road/Buses</x:v>
+      </x:c>
+      <x:c r="B107" s="28" t="str">
+        <x:v>15.02.02.01 Buses</x:v>
+      </x:c>
+      <x:c r="C107" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="28" t="str">
+        <x:v>Passenger road/Buses/BEV</x:v>
+      </x:c>
+      <x:c r="B108" s="28" t="str">
+        <x:v>15.02.02.01.01 BEV</x:v>
+      </x:c>
+      <x:c r="C108" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="28" t="str">
+        <x:v>Passenger road/Buses/FCEV</x:v>
+      </x:c>
+      <x:c r="B109" s="28" t="str">
+        <x:v>15.02.02.01.02 FCEV</x:v>
+      </x:c>
+      <x:c r="C109" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="28" t="str">
+        <x:v>Passenger road/Buses/ICE</x:v>
+      </x:c>
+      <x:c r="B110" s="28" t="str">
+        <x:v>15.02.02.01.03 ICE</x:v>
+      </x:c>
+      <x:c r="C110" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="28" t="str">
+        <x:v>Passenger road/LPVs</x:v>
+      </x:c>
+      <x:c r="B111" s="28" t="str">
+        <x:v>15.02.02.02 LPVs</x:v>
+      </x:c>
+      <x:c r="C111" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="28" t="str">
+        <x:v>Passenger road/LPVs/BEV large</x:v>
+      </x:c>
+      <x:c r="B112" s="28" t="str">
+        <x:v>15.02.02.02.01 BEV large</x:v>
+      </x:c>
+      <x:c r="C112" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="28" t="str">
+        <x:v>Passenger road/LPVs/BEV medium</x:v>
+      </x:c>
+      <x:c r="B113" s="28" t="str">
+        <x:v>15.02.02.02.02 BEV medium</x:v>
+      </x:c>
+      <x:c r="C113" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="28" t="str">
+        <x:v>Passenger road/LPVs/BEV small</x:v>
+      </x:c>
+      <x:c r="B114" s="28" t="str">
+        <x:v>15.02.02.02.03 BEV small</x:v>
+      </x:c>
+      <x:c r="C114" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="28" t="str">
+        <x:v>Passenger road/LPVs/EREV large</x:v>
+      </x:c>
+      <x:c r="B115" s="28" t="str">
+        <x:v>15.02.02.02.04 EREV large</x:v>
+      </x:c>
+      <x:c r="C115" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="28" t="str">
+        <x:v>Passenger road/LPVs/EREV medium</x:v>
+      </x:c>
+      <x:c r="B116" s="28" t="str">
+        <x:v>15.02.02.02.05 EREV medium</x:v>
+      </x:c>
+      <x:c r="C116" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="28" t="str">
+        <x:v>Passenger road/LPVs/EREV small</x:v>
+      </x:c>
+      <x:c r="B117" s="28" t="str">
+        <x:v>15.02.02.02.06 EREV small</x:v>
+      </x:c>
+      <x:c r="C117" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="28" t="str">
+        <x:v>Passenger road/LPVs/HEV large</x:v>
+      </x:c>
+      <x:c r="B118" s="28" t="str">
+        <x:v>15.02.02.02.07 HEV large</x:v>
+      </x:c>
+      <x:c r="C118" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="28" t="str">
+        <x:v>Passenger road/LPVs/HEV medium</x:v>
+      </x:c>
+      <x:c r="B119" s="28" t="str">
+        <x:v>15.02.02.02.08 HEV medium</x:v>
+      </x:c>
+      <x:c r="C119" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="28" t="str">
+        <x:v>Passenger road/LPVs/HEV small</x:v>
+      </x:c>
+      <x:c r="B120" s="28" t="str">
+        <x:v>15.02.02.02.09 HEV small</x:v>
+      </x:c>
+      <x:c r="C120" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="28" t="str">
+        <x:v>Passenger road/LPVs/ICE large</x:v>
+      </x:c>
+      <x:c r="B121" s="28" t="str">
+        <x:v>15.02.02.02.10 ICE large</x:v>
+      </x:c>
+      <x:c r="C121" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="28" t="str">
+        <x:v>Passenger road/LPVs/ICE medium</x:v>
+      </x:c>
+      <x:c r="B122" s="28" t="str">
+        <x:v>15.02.02.02.11 ICE medium</x:v>
+      </x:c>
+      <x:c r="C122" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="28" t="str">
+        <x:v>Passenger road/LPVs/ICE small</x:v>
+      </x:c>
+      <x:c r="B123" s="28" t="str">
+        <x:v>15.02.02.02.12 ICE small</x:v>
+      </x:c>
+      <x:c r="C123" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="28" t="str">
+        <x:v>Passenger road/LPVs/PHEV large</x:v>
+      </x:c>
+      <x:c r="B124" s="28" t="str">
+        <x:v>15.02.02.02.13 PHEV large</x:v>
+      </x:c>
+      <x:c r="C124" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="28" t="str">
+        <x:v>Passenger road/LPVs/PHEV medium</x:v>
+      </x:c>
+      <x:c r="B125" s="28" t="str">
+        <x:v>15.02.02.02.14 PHEV medium</x:v>
+      </x:c>
+      <x:c r="C125" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="28" t="str">
+        <x:v>Passenger road/LPVs/PHEV small</x:v>
+      </x:c>
+      <x:c r="B126" s="28" t="str">
+        <x:v>15.02.02.02.15 PHEV small</x:v>
+      </x:c>
+      <x:c r="C126" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="28" t="str">
+        <x:v>Passenger road/Motorcycles</x:v>
+      </x:c>
+      <x:c r="B127" s="28" t="str">
+        <x:v>15.02.02.03 Motorcycles</x:v>
+      </x:c>
+      <x:c r="C127" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="28" t="str">
+        <x:v>Passenger road/Motorcycles/BEV</x:v>
+      </x:c>
+      <x:c r="B128" s="28" t="str">
+        <x:v>15.02.02.03.01 BEV</x:v>
+      </x:c>
+      <x:c r="C128" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="28" t="str">
+        <x:v>Passenger road/Motorcycles/ICE</x:v>
+      </x:c>
+      <x:c r="B129" s="28" t="str">
+        <x:v>15.02.02.03.02 ICE</x:v>
+      </x:c>
+      <x:c r="C129" s="28" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="28" t="str">
+        <x:v>Patent fuel plants/Patent fuel plants</x:v>
+      </x:c>
+      <x:c r="B130" s="28" t="str">
+        <x:v>09.08.03 Patent fuel plants</x:v>
+      </x:c>
+      <x:c r="C130" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="28" t="str">
+        <x:v>Petrochemical industry/Petrochemical industry</x:v>
+      </x:c>
+      <x:c r="B131" s="28" t="str">
+        <x:v>09.09 Petrochemical industry</x:v>
+      </x:c>
+      <x:c r="C131" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="28" t="str">
+        <x:v>Power</x:v>
+      </x:c>
+      <x:c r="B132" s="28" t="str">
+        <x:v>09.01-09.02 Power sector</x:v>
+      </x:c>
+      <x:c r="C132" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="28" t="str">
+        <x:v>Production</x:v>
+      </x:c>
+      <x:c r="B133" s="28" t="str">
+        <x:v>01 Production</x:v>
+      </x:c>
+      <x:c r="C133" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="28" t="str">
+        <x:v>Road</x:v>
+      </x:c>
+      <x:c r="B134" s="28" t="str">
+        <x:v>15.02 Road</x:v>
+      </x:c>
+      <x:c r="C134" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="28" t="str">
+        <x:v>Statistical Differences</x:v>
+      </x:c>
+      <x:c r="B135" s="28" t="str">
+        <x:v>11 Statistical discrepancy</x:v>
+      </x:c>
+      <x:c r="C135" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="28" t="str">
+        <x:v>Stock Changes</x:v>
+      </x:c>
+      <x:c r="B136" s="28" t="str">
+        <x:v>06 Stock changes</x:v>
+      </x:c>
+      <x:c r="C136" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="28" t="str">
+        <x:v>Total Primary Supply</x:v>
+      </x:c>
+      <x:c r="B137" s="28" t="str">
+        <x:v>07 Total primary energy supply</x:v>
+      </x:c>
+      <x:c r="C137" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="28" t="str">
+        <x:v>Total final consumption</x:v>
+      </x:c>
+      <x:c r="B138" s="28" t="str">
+        <x:v>12 Total final consumption</x:v>
+      </x:c>
+      <x:c r="C138" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="28" t="str">
+        <x:v>Total final energy consumption</x:v>
+      </x:c>
+      <x:c r="B139" s="28" t="str">
+        <x:v>13 Total final energy consumption</x:v>
+      </x:c>
+      <x:c r="C139" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="28" t="str">
+        <x:v>Total transformation - no transfers</x:v>
+      </x:c>
+      <x:c r="B140" s="28" t="str">
+        <x:v>09 Total transformation sector</x:v>
+      </x:c>
+      <x:c r="C140" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="28" t="str">
+        <x:v>Transfers</x:v>
+      </x:c>
+      <x:c r="B141" s="28" t="str">
+        <x:v>08 Transfers</x:v>
+      </x:c>
+      <x:c r="C141" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="28" t="str">
+        <x:v>Transmission and Distribution</x:v>
+      </x:c>
+      <x:c r="B142" s="28" t="str">
+        <x:v>10.02 Transmission and distribution losses</x:v>
+      </x:c>
+      <x:c r="C142" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="28" t="str">
+        <x:v>Transport</x:v>
+      </x:c>
+      <x:c r="B143" s="28" t="str">
+        <x:v>15 Transport sector</x:v>
+      </x:c>
+      <x:c r="C143" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="28" t="str">
+        <x:v>Transport non road</x:v>
+      </x:c>
+      <x:c r="B144" s="28" t="str">
+        <x:v>15.01,15.03-15.06 Transport non-road</x:v>
+      </x:c>
+      <x:c r="C144" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="28" t="str">
+        <x:v>Transport non road/Freight non road/Air</x:v>
+      </x:c>
+      <x:c r="B145" s="28" t="str">
+        <x:v>15.01 Domestic air transport</x:v>
+      </x:c>
+      <x:c r="C145" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="28" t="str">
+        <x:v>Transport non road/Freight non road/Rail</x:v>
+      </x:c>
+      <x:c r="B146" s="28" t="str">
+        <x:v>15.03 Rail</x:v>
+      </x:c>
+      <x:c r="C146" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="28" t="str">
+        <x:v>Transport non road/Freight non road/Shipping</x:v>
+      </x:c>
+      <x:c r="B147" s="28" t="str">
+        <x:v>15.04 Domestic navigation</x:v>
+      </x:c>
+      <x:c r="C147" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="28" t="str">
+        <x:v>Transport non road/International transport/Air</x:v>
+      </x:c>
+      <x:c r="B148" s="28" t="str">
+        <x:v>05 International aviation bunkers</x:v>
+      </x:c>
+      <x:c r="C148" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="28" t="str">
+        <x:v>Transport non road/International transport/Shipping</x:v>
+      </x:c>
+      <x:c r="B149" s="28" t="str">
+        <x:v>04 International marine bunkers</x:v>
+      </x:c>
+      <x:c r="C149" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="28" t="str">
+        <x:v>Transport non road/Nonspecified transport</x:v>
+      </x:c>
+      <x:c r="B150" s="28" t="str">
+        <x:v>15.02 Road</x:v>
+      </x:c>
+      <x:c r="C150" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="28" t="str">
+        <x:v>Transport non road/Nonspecified transport</x:v>
+      </x:c>
+      <x:c r="B151" s="28" t="str">
+        <x:v>15.03 Rail</x:v>
+      </x:c>
+      <x:c r="C151" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="28" t="str">
+        <x:v>Transport non road/Nonspecified transport</x:v>
+      </x:c>
+      <x:c r="B152" s="28" t="str">
+        <x:v>15.06 Non-specified transport</x:v>
+      </x:c>
+      <x:c r="C152" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="28" t="str">
+        <x:v>Transport non road/Passenger non road/Air</x:v>
+      </x:c>
+      <x:c r="B153" s="28" t="str">
+        <x:v>15.01 Domestic air transport</x:v>
+      </x:c>
+      <x:c r="C153" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" s="28" t="str">
+        <x:v>Transport non road/Passenger non road/Rail</x:v>
+      </x:c>
+      <x:c r="B154" s="28" t="str">
+        <x:v>15.03 Rail</x:v>
+      </x:c>
+      <x:c r="C154" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" s="28" t="str">
         <x:v>Transport non road/Passenger non road/Shipping</x:v>
       </x:c>
-      <x:c r="B98" s="28" t="str">
+      <x:c r="B155" s="28" t="str">
         <x:v>15.04 Domestic navigation</x:v>
       </x:c>
-      <x:c r="C98" s="28" t="str">
-        <x:v>BOTH</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99">
-      <x:c r="A99" s="29" t="str">
+      <x:c r="C155" s="28" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" s="29" t="str">
         <x:v>Transport non road/Pipeline transport</x:v>
       </x:c>
-      <x:c r="B99" s="29" t="str">
+      <x:c r="B156" s="29" t="str">
         <x:v>15.05 Pipeline transport</x:v>
       </x:c>
-      <x:c r="C99" s="29" t="str">
+      <x:c r="C156" s="29" t="str">
         <x:v>BOTH</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" allowBlank="0" showDropDown="0" sqref="C2:C99">
+    <x:dataValidation type="list" allowBlank="0" showDropDown="0" sqref="C2:C156">
       <x:formula1>"BOTH,ESTO,ESTO_EXTENDED"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -17016,7 +17643,7 @@
         <x:v>Anthracite</x:v>
       </x:c>
       <x:c r="B4" s="28" t="str">
-        <x:v>01.03 Sub-bituminous coal</x:v>
+        <x:v>01.04 Anthracite</x:v>
       </x:c>
       <x:c r="C4" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17030,7 +17657,7 @@
         <x:v>01.04 Anthracite</x:v>
       </x:c>
       <x:c r="C5" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -17038,7 +17665,7 @@
         <x:v>Aviation gasoline</x:v>
       </x:c>
       <x:c r="B6" s="28" t="str">
-        <x:v>07.01 Motor gasoline</x:v>
+        <x:v>07.02 Aviation gasoline</x:v>
       </x:c>
       <x:c r="C6" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17046,10 +17673,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="28" t="str">
-        <x:v>Aviation gasoline</x:v>
+        <x:v>BKB and PB</x:v>
       </x:c>
       <x:c r="B7" s="28" t="str">
-        <x:v>07.02 Aviation gasoline</x:v>
+        <x:v>02.08 BKB/PB</x:v>
       </x:c>
       <x:c r="C7" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17060,18 +17687,18 @@
         <x:v>BKB and PB</x:v>
       </x:c>
       <x:c r="B8" s="28" t="str">
-        <x:v>02.07 Coal tar</x:v>
+        <x:v>02.08 BKB/PB</x:v>
       </x:c>
       <x:c r="C8" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="28" t="str">
-        <x:v>BKB and PB</x:v>
+        <x:v>Bagasse</x:v>
       </x:c>
       <x:c r="B9" s="28" t="str">
-        <x:v>02.08 BKB/PB</x:v>
+        <x:v>15.02 Bagasse</x:v>
       </x:c>
       <x:c r="C9" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17079,10 +17706,10 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="28" t="str">
-        <x:v>Bagasse</x:v>
+        <x:v>Bio jet kerosene</x:v>
       </x:c>
       <x:c r="B10" s="28" t="str">
-        <x:v>04 Peat products</x:v>
+        <x:v>16.07 Bio jet kerosene</x:v>
       </x:c>
       <x:c r="C10" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17090,10 +17717,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="28" t="str">
-        <x:v>Bagasse</x:v>
+        <x:v>Biodiesel</x:v>
       </x:c>
       <x:c r="B11" s="28" t="str">
-        <x:v>15.02 Bagasse</x:v>
+        <x:v>16.06 Biodiesel</x:v>
       </x:c>
       <x:c r="C11" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17101,21 +17728,21 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="28" t="str">
-        <x:v>Bio jet kerosene</x:v>
+        <x:v>Biodiesel</x:v>
       </x:c>
       <x:c r="B12" s="28" t="str">
-        <x:v>16.07 Bio jet kerosene</x:v>
+        <x:v>16.06 Biodiesel</x:v>
       </x:c>
       <x:c r="C12" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="28" t="str">
-        <x:v>Biodiesel</x:v>
+        <x:v>Biogas</x:v>
       </x:c>
       <x:c r="B13" s="28" t="str">
-        <x:v>16.05 Biogasoline</x:v>
+        <x:v>16.01 Biogas</x:v>
       </x:c>
       <x:c r="C13" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17123,21 +17750,21 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="28" t="str">
-        <x:v>Biodiesel</x:v>
+        <x:v>Biogas</x:v>
       </x:c>
       <x:c r="B14" s="28" t="str">
-        <x:v>16.06 Biodiesel</x:v>
+        <x:v>16.01 Biogas</x:v>
       </x:c>
       <x:c r="C14" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="28" t="str">
-        <x:v>Biogas</x:v>
+        <x:v>Biogasoline</x:v>
       </x:c>
       <x:c r="B15" s="28" t="str">
-        <x:v>15.05 Other biomass</x:v>
+        <x:v>16.05 Biogasoline</x:v>
       </x:c>
       <x:c r="C15" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17145,21 +17772,21 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="28" t="str">
-        <x:v>Biogas</x:v>
+        <x:v>Biogasoline</x:v>
       </x:c>
       <x:c r="B16" s="28" t="str">
-        <x:v>16.01 Biogas</x:v>
+        <x:v>16.05 Biogasoline</x:v>
       </x:c>
       <x:c r="C16" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="28" t="str">
-        <x:v>Biogasoline</x:v>
+        <x:v>Bitumen</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>16.04 Municipal solid waste (non-renewable)</x:v>
+        <x:v>07.14 Bitumen</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17167,10 +17794,10 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="28" t="str">
-        <x:v>Biogasoline</x:v>
+        <x:v>Black liquor</x:v>
       </x:c>
       <x:c r="B18" s="28" t="str">
-        <x:v>16.05 Biogasoline</x:v>
+        <x:v>15.04 Black liquor</x:v>
       </x:c>
       <x:c r="C18" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17178,10 +17805,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="28" t="str">
-        <x:v>Bitumen</x:v>
+        <x:v>Blast furnace gas</x:v>
       </x:c>
       <x:c r="B19" s="28" t="str">
-        <x:v>07.14 Bitumen</x:v>
+        <x:v>02.04 Blast furnace gas</x:v>
       </x:c>
       <x:c r="C19" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17189,21 +17816,21 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="28" t="str">
-        <x:v>Black liquor</x:v>
+        <x:v>Blast furnace gas</x:v>
       </x:c>
       <x:c r="B20" s="28" t="str">
-        <x:v>15.04 Black liquor</x:v>
+        <x:v>02.04 Blast furnace gas</x:v>
       </x:c>
       <x:c r="C20" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="28" t="str">
-        <x:v>Blast furnace gas</x:v>
+        <x:v>Charcoal</x:v>
       </x:c>
       <x:c r="B21" s="28" t="str">
-        <x:v>02.03 Coke oven gas</x:v>
+        <x:v>15.03 Charcoal</x:v>
       </x:c>
       <x:c r="C21" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17211,10 +17838,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="28" t="str">
-        <x:v>Blast furnace gas</x:v>
+        <x:v>Coal nonspecified</x:v>
       </x:c>
       <x:c r="B22" s="28" t="str">
-        <x:v>02.04 Blast furnace gas</x:v>
+        <x:v>01.99 Coal nonspecified</x:v>
       </x:c>
       <x:c r="C22" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17222,10 +17849,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="28" t="str">
-        <x:v>Charcoal</x:v>
+        <x:v>Coal tar</x:v>
       </x:c>
       <x:c r="B23" s="28" t="str">
-        <x:v>15.01 Fuelwood &amp; woodwaste</x:v>
+        <x:v>02.07 Coal tar</x:v>
       </x:c>
       <x:c r="C23" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17233,21 +17860,21 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="28" t="str">
-        <x:v>Charcoal</x:v>
+        <x:v>Coal tar</x:v>
       </x:c>
       <x:c r="B24" s="28" t="str">
-        <x:v>15.03 Charcoal</x:v>
+        <x:v>02.07 Coal tar</x:v>
       </x:c>
       <x:c r="C24" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="28" t="str">
-        <x:v>Coal nonspecified</x:v>
+        <x:v>Coke oven coke</x:v>
       </x:c>
       <x:c r="B25" s="28" t="str">
-        <x:v>01.99 Coal nonspecified</x:v>
+        <x:v>02.01 Coke oven coke</x:v>
       </x:c>
       <x:c r="C25" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17255,21 +17882,21 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="28" t="str">
-        <x:v>Coal tar</x:v>
+        <x:v>Coke oven coke</x:v>
       </x:c>
       <x:c r="B26" s="28" t="str">
-        <x:v>02.06 Patent fuel</x:v>
+        <x:v>02.01 Coke oven coke</x:v>
       </x:c>
       <x:c r="C26" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="28" t="str">
-        <x:v>Coal tar</x:v>
+        <x:v>Coke oven gas</x:v>
       </x:c>
       <x:c r="B27" s="28" t="str">
-        <x:v>02.07 Coal tar</x:v>
+        <x:v>02.03 Coke oven gas</x:v>
       </x:c>
       <x:c r="C27" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17277,21 +17904,21 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="28" t="str">
-        <x:v>Coke oven coke</x:v>
+        <x:v>Coke oven gas</x:v>
       </x:c>
       <x:c r="B28" s="28" t="str">
-        <x:v>01.05 Lignite</x:v>
+        <x:v>02.03 Coke oven gas</x:v>
       </x:c>
       <x:c r="C28" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="28" t="str">
-        <x:v>Coke oven coke</x:v>
+        <x:v>Coking coal</x:v>
       </x:c>
       <x:c r="B29" s="28" t="str">
-        <x:v>02.01 Coke oven coke</x:v>
+        <x:v>01.01 Coking coal</x:v>
       </x:c>
       <x:c r="C29" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17299,21 +17926,21 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="28" t="str">
-        <x:v>Coke oven gas</x:v>
+        <x:v>Coking coal</x:v>
       </x:c>
       <x:c r="B30" s="28" t="str">
-        <x:v>02.01 Coke oven coke</x:v>
+        <x:v>01.01 Coking coal</x:v>
       </x:c>
       <x:c r="C30" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="28" t="str">
-        <x:v>Coke oven gas</x:v>
+        <x:v>Crude oil</x:v>
       </x:c>
       <x:c r="B31" s="28" t="str">
-        <x:v>02.03 Coke oven gas</x:v>
+        <x:v>06.01 Crude oil</x:v>
       </x:c>
       <x:c r="C31" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17321,10 +17948,10 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="28" t="str">
-        <x:v>Coking coal</x:v>
+        <x:v>Efuel</x:v>
       </x:c>
       <x:c r="B32" s="28" t="str">
-        <x:v>01.01 Coking coal</x:v>
+        <x:v>16.11 E-fuel</x:v>
       </x:c>
       <x:c r="C32" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17332,21 +17959,21 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="28" t="str">
-        <x:v>Crude oil</x:v>
+        <x:v>Efuel</x:v>
       </x:c>
       <x:c r="B33" s="28" t="str">
-        <x:v>06.01 Crude oil</x:v>
+        <x:v>16.11 E-fuel</x:v>
       </x:c>
       <x:c r="C33" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="28" t="str">
-        <x:v>Efuel</x:v>
+        <x:v>Electricity</x:v>
       </x:c>
       <x:c r="B34" s="28" t="str">
-        <x:v>16.11 E-fuel</x:v>
+        <x:v>17 Electricity</x:v>
       </x:c>
       <x:c r="C34" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17357,18 +17984,18 @@
         <x:v>Electricity</x:v>
       </x:c>
       <x:c r="B35" s="28" t="str">
-        <x:v>16.12 Hydrogen</x:v>
+        <x:v>17 Electricity</x:v>
       </x:c>
       <x:c r="C35" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="28" t="str">
-        <x:v>Electricity</x:v>
+        <x:v>Ethane</x:v>
       </x:c>
       <x:c r="B36" s="28" t="str">
-        <x:v>17 Electricity</x:v>
+        <x:v>07.11 Ethane</x:v>
       </x:c>
       <x:c r="C36" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17376,32 +18003,32 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="28" t="str">
-        <x:v>Electricity</x:v>
+        <x:v>Fuel oil</x:v>
       </x:c>
       <x:c r="B37" s="28" t="str">
-        <x:v>17 Electricity</x:v>
+        <x:v>07.08 Fuel oil</x:v>
       </x:c>
       <x:c r="C37" s="28" t="str">
-        <x:v>ESTO_EXTENDED</x:v>
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="28" t="str">
-        <x:v>Ethane</x:v>
+        <x:v>Fuel oil</x:v>
       </x:c>
       <x:c r="B38" s="28" t="str">
-        <x:v>07.11 Ethane</x:v>
+        <x:v>07.08 Fuel oil</x:v>
       </x:c>
       <x:c r="C38" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="28" t="str">
-        <x:v>Fuel oil</x:v>
+        <x:v>Fuelwood and woodwaste</x:v>
       </x:c>
       <x:c r="B39" s="28" t="str">
-        <x:v>07.07 Gas/diesel oil</x:v>
+        <x:v>15.01 Fuelwood &amp; woodwaste</x:v>
       </x:c>
       <x:c r="C39" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17409,10 +18036,10 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="28" t="str">
-        <x:v>Fuel oil</x:v>
+        <x:v>Gas and diesel oil</x:v>
       </x:c>
       <x:c r="B40" s="28" t="str">
-        <x:v>07.08 Fuel oil</x:v>
+        <x:v>07.07 Gas/diesel oil</x:v>
       </x:c>
       <x:c r="C40" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17420,21 +18047,21 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="28" t="str">
-        <x:v>Fuelwood and woodwaste</x:v>
+        <x:v>Gas and diesel oil</x:v>
       </x:c>
       <x:c r="B41" s="28" t="str">
-        <x:v>12.99 Solar nonspecified</x:v>
+        <x:v>07.07 Gas/diesel oil</x:v>
       </x:c>
       <x:c r="C41" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="28" t="str">
-        <x:v>Fuelwood and woodwaste</x:v>
+        <x:v>Gas coke</x:v>
       </x:c>
       <x:c r="B42" s="28" t="str">
-        <x:v>15.01 Fuelwood &amp; woodwaste</x:v>
+        <x:v>02.02 Gas coke</x:v>
       </x:c>
       <x:c r="C42" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17442,10 +18069,10 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="28" t="str">
-        <x:v>Gas and diesel oil</x:v>
+        <x:v>Gas nonspecified</x:v>
       </x:c>
       <x:c r="B43" s="28" t="str">
-        <x:v>07.06 Kerosene</x:v>
+        <x:v>08.99 Gas nonspecified</x:v>
       </x:c>
       <x:c r="C43" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17453,10 +18080,10 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="28" t="str">
-        <x:v>Gas and diesel oil</x:v>
+        <x:v>Gas works gas</x:v>
       </x:c>
       <x:c r="B44" s="28" t="str">
-        <x:v>07.07 Gas/diesel oil</x:v>
+        <x:v>08.03 Gas works gas</x:v>
       </x:c>
       <x:c r="C44" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17464,21 +18091,21 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="28" t="str">
-        <x:v>Gas coke</x:v>
+        <x:v>Gas works gas</x:v>
       </x:c>
       <x:c r="B45" s="28" t="str">
-        <x:v>02.02 Gas coke</x:v>
+        <x:v>08.03 Gas works gas</x:v>
       </x:c>
       <x:c r="C45" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="28" t="str">
-        <x:v>Gas nonspecified</x:v>
+        <x:v>Gasoline type jet fuel</x:v>
       </x:c>
       <x:c r="B46" s="28" t="str">
-        <x:v>08.99 Gas nonspecified</x:v>
+        <x:v>07.04 Gasoline type jet fuel</x:v>
       </x:c>
       <x:c r="C46" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17486,10 +18113,10 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="28" t="str">
-        <x:v>Gas works gas</x:v>
+        <x:v>Geothermal</x:v>
       </x:c>
       <x:c r="B47" s="28" t="str">
-        <x:v>08.01 Natural gas</x:v>
+        <x:v>11 Geothermal</x:v>
       </x:c>
       <x:c r="C47" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17497,10 +18124,10 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="28" t="str">
-        <x:v>Gas works gas</x:v>
+        <x:v>Heat</x:v>
       </x:c>
       <x:c r="B48" s="28" t="str">
-        <x:v>08.03 Gas works gas</x:v>
+        <x:v>18 Heat</x:v>
       </x:c>
       <x:c r="C48" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17508,21 +18135,21 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="28" t="str">
-        <x:v>Gasoline type jet fuel</x:v>
+        <x:v>Heat</x:v>
       </x:c>
       <x:c r="B49" s="28" t="str">
-        <x:v>07.04 Gasoline type jet fuel</x:v>
+        <x:v>18 Heat</x:v>
       </x:c>
       <x:c r="C49" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="28" t="str">
-        <x:v>Geothermal</x:v>
+        <x:v>Hydro</x:v>
       </x:c>
       <x:c r="B50" s="28" t="str">
-        <x:v>08.03 Gas works gas</x:v>
+        <x:v>10 Hydro</x:v>
       </x:c>
       <x:c r="C50" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17530,10 +18157,10 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="28" t="str">
-        <x:v>Geothermal</x:v>
+        <x:v>Hydrogen</x:v>
       </x:c>
       <x:c r="B51" s="28" t="str">
-        <x:v>11 Geothermal</x:v>
+        <x:v>16.12 Hydrogen</x:v>
       </x:c>
       <x:c r="C51" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17541,21 +18168,21 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="28" t="str">
-        <x:v>Heat</x:v>
+        <x:v>Hydrogen</x:v>
       </x:c>
       <x:c r="B52" s="28" t="str">
-        <x:v>17 Electricity</x:v>
+        <x:v>16.12 Hydrogen</x:v>
       </x:c>
       <x:c r="C52" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="28" t="str">
-        <x:v>Heat</x:v>
+        <x:v>Industrial waste</x:v>
       </x:c>
       <x:c r="B53" s="28" t="str">
-        <x:v>18 Heat</x:v>
+        <x:v>16.02 Industrial waste</x:v>
       </x:c>
       <x:c r="C53" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17563,21 +18190,21 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="28" t="str">
-        <x:v>Hydro</x:v>
+        <x:v>Industrial waste</x:v>
       </x:c>
       <x:c r="B54" s="28" t="str">
-        <x:v>10 Hydro</x:v>
+        <x:v>16.02 Industrial waste</x:v>
       </x:c>
       <x:c r="C54" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="28" t="str">
-        <x:v>Hydrogen</x:v>
+        <x:v>Kerosene</x:v>
       </x:c>
       <x:c r="B55" s="28" t="str">
-        <x:v>16.06 Biodiesel</x:v>
+        <x:v>07.06 Kerosene</x:v>
       </x:c>
       <x:c r="C55" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17585,21 +18212,21 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="28" t="str">
-        <x:v>Hydrogen</x:v>
+        <x:v>Kerosene</x:v>
       </x:c>
       <x:c r="B56" s="28" t="str">
-        <x:v>16.12 Hydrogen</x:v>
+        <x:v>07.06 Kerosene</x:v>
       </x:c>
       <x:c r="C56" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="28" t="str">
-        <x:v>Industrial waste</x:v>
+        <x:v>Kerosene type jet fuel</x:v>
       </x:c>
       <x:c r="B57" s="28" t="str">
-        <x:v>16.01 Biogas</x:v>
+        <x:v>07.05 Kerosene type jet fuel</x:v>
       </x:c>
       <x:c r="C57" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17607,21 +18234,21 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="28" t="str">
-        <x:v>Industrial waste</x:v>
+        <x:v>Kerosene type jet fuel</x:v>
       </x:c>
       <x:c r="B58" s="28" t="str">
-        <x:v>16.02 Industrial waste</x:v>
+        <x:v>07.05 Kerosene type jet fuel</x:v>
       </x:c>
       <x:c r="C58" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="28" t="str">
-        <x:v>Kerosene</x:v>
+        <x:v>LNG</x:v>
       </x:c>
       <x:c r="B59" s="28" t="str">
-        <x:v>07.05 Kerosene type jet fuel</x:v>
+        <x:v>08.02 LNG</x:v>
       </x:c>
       <x:c r="C59" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17629,10 +18256,10 @@
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="28" t="str">
-        <x:v>Kerosene</x:v>
+        <x:v>LPG</x:v>
       </x:c>
       <x:c r="B60" s="28" t="str">
-        <x:v>07.06 Kerosene</x:v>
+        <x:v>07.09 LPG</x:v>
       </x:c>
       <x:c r="C60" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17640,21 +18267,21 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="28" t="str">
-        <x:v>Kerosene type jet fuel</x:v>
+        <x:v>LPG</x:v>
       </x:c>
       <x:c r="B61" s="28" t="str">
-        <x:v>07.02 Aviation gasoline</x:v>
+        <x:v>07.09 LPG</x:v>
       </x:c>
       <x:c r="C61" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="28" t="str">
-        <x:v>Kerosene type jet fuel</x:v>
+        <x:v>Lignite</x:v>
       </x:c>
       <x:c r="B62" s="28" t="str">
-        <x:v>07.05 Kerosene type jet fuel</x:v>
+        <x:v>01.05 Lignite</x:v>
       </x:c>
       <x:c r="C62" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17662,10 +18289,10 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="28" t="str">
-        <x:v>LNG</x:v>
+        <x:v>Lubricants</x:v>
       </x:c>
       <x:c r="B63" s="28" t="str">
-        <x:v>08.02 LNG</x:v>
+        <x:v>07.13 Lubricants</x:v>
       </x:c>
       <x:c r="C63" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17673,10 +18300,10 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="28" t="str">
-        <x:v>LPG</x:v>
+        <x:v>Motor gasoline</x:v>
       </x:c>
       <x:c r="B64" s="28" t="str">
-        <x:v>07.08 Fuel oil</x:v>
+        <x:v>07.01 Motor gasoline</x:v>
       </x:c>
       <x:c r="C64" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17684,21 +18311,21 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="28" t="str">
-        <x:v>LPG</x:v>
+        <x:v>Motor gasoline</x:v>
       </x:c>
       <x:c r="B65" s="28" t="str">
-        <x:v>07.09 LPG</x:v>
+        <x:v>07.01 Motor gasoline</x:v>
       </x:c>
       <x:c r="C65" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="28" t="str">
-        <x:v>Lignite</x:v>
+        <x:v>Municipal solid waste non renewable</x:v>
       </x:c>
       <x:c r="B66" s="28" t="str">
-        <x:v>01.04 Anthracite</x:v>
+        <x:v>16.04 Municipal solid waste (non-renewable)</x:v>
       </x:c>
       <x:c r="C66" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17706,21 +18333,21 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="28" t="str">
-        <x:v>Lignite</x:v>
+        <x:v>Municipal solid waste non renewable</x:v>
       </x:c>
       <x:c r="B67" s="28" t="str">
-        <x:v>01.05 Lignite</x:v>
+        <x:v>16.04 Municipal solid waste (non-renewable)</x:v>
       </x:c>
       <x:c r="C67" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="28" t="str">
-        <x:v>Lubricants</x:v>
+        <x:v>Municipal solid waste renewable</x:v>
       </x:c>
       <x:c r="B68" s="28" t="str">
-        <x:v>07.13 Lubricants</x:v>
+        <x:v>16.03 Municipal solid waste (renewable)</x:v>
       </x:c>
       <x:c r="C68" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17728,21 +18355,21 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="28" t="str">
-        <x:v>Motor gasoline</x:v>
+        <x:v>Municipal solid waste renewable</x:v>
       </x:c>
       <x:c r="B69" s="28" t="str">
-        <x:v>02.08 BKB/PB</x:v>
+        <x:v>16.03 Municipal solid waste (renewable)</x:v>
       </x:c>
       <x:c r="C69" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="28" t="str">
-        <x:v>Motor gasoline</x:v>
+        <x:v>Naphtha</x:v>
       </x:c>
       <x:c r="B70" s="28" t="str">
-        <x:v>07.01 Motor gasoline</x:v>
+        <x:v>07.03 Naphtha</x:v>
       </x:c>
       <x:c r="C70" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17750,10 +18377,10 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="28" t="str">
-        <x:v>Municipal solid waste non renewable</x:v>
+        <x:v>Natural gas</x:v>
       </x:c>
       <x:c r="B71" s="28" t="str">
-        <x:v>16.03 Municipal solid waste (renewable)</x:v>
+        <x:v>08.01 Natural gas</x:v>
       </x:c>
       <x:c r="C71" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17761,21 +18388,21 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="28" t="str">
-        <x:v>Municipal solid waste non renewable</x:v>
+        <x:v>Natural gas</x:v>
       </x:c>
       <x:c r="B72" s="28" t="str">
-        <x:v>16.04 Municipal solid waste (non-renewable)</x:v>
+        <x:v>08.01 Natural gas</x:v>
       </x:c>
       <x:c r="C72" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="28" t="str">
-        <x:v>Municipal solid waste renewable</x:v>
+        <x:v>Natural gas liquids</x:v>
       </x:c>
       <x:c r="B73" s="28" t="str">
-        <x:v>16.02 Industrial waste</x:v>
+        <x:v>06.02 Natural gas liquids</x:v>
       </x:c>
       <x:c r="C73" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17783,10 +18410,10 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="28" t="str">
-        <x:v>Municipal solid waste renewable</x:v>
+        <x:v>Nuclear</x:v>
       </x:c>
       <x:c r="B74" s="28" t="str">
-        <x:v>16.03 Municipal solid waste (renewable)</x:v>
+        <x:v>09 Nuclear</x:v>
       </x:c>
       <x:c r="C74" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17794,10 +18421,10 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="28" t="str">
-        <x:v>Naphtha</x:v>
+        <x:v>Oil shale and oil sands</x:v>
       </x:c>
       <x:c r="B75" s="28" t="str">
-        <x:v>07.03 Naphtha</x:v>
+        <x:v>05 Oil shale and oil sands</x:v>
       </x:c>
       <x:c r="C75" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17805,10 +18432,10 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="28" t="str">
-        <x:v>Natural gas</x:v>
+        <x:v>Other biomass</x:v>
       </x:c>
       <x:c r="B76" s="28" t="str">
-        <x:v>07.09 LPG</x:v>
+        <x:v>15.05 Other biomass</x:v>
       </x:c>
       <x:c r="C76" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17816,21 +18443,21 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="28" t="str">
-        <x:v>Natural gas</x:v>
+        <x:v>Other biomass</x:v>
       </x:c>
       <x:c r="B77" s="28" t="str">
-        <x:v>08.01 Natural gas</x:v>
+        <x:v>15.05 Other biomass</x:v>
       </x:c>
       <x:c r="C77" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="28" t="str">
-        <x:v>Natural gas liquids</x:v>
+        <x:v>Other bituminous coal</x:v>
       </x:c>
       <x:c r="B78" s="28" t="str">
-        <x:v>06.02 Natural gas liquids</x:v>
+        <x:v>01.02 Other bituminous coal</x:v>
       </x:c>
       <x:c r="C78" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17838,21 +18465,21 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="28" t="str">
-        <x:v>Nuclear</x:v>
+        <x:v>Other bituminous coal</x:v>
       </x:c>
       <x:c r="B79" s="28" t="str">
-        <x:v>09 Nuclear</x:v>
+        <x:v>01.02 Other bituminous coal</x:v>
       </x:c>
       <x:c r="C79" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="28" t="str">
-        <x:v>Oil shale and oil sands</x:v>
+        <x:v>Other hydrocarbons</x:v>
       </x:c>
       <x:c r="B80" s="28" t="str">
-        <x:v>05 Oil shale and oil sands</x:v>
+        <x:v>06.05 Other hydrocarbons</x:v>
       </x:c>
       <x:c r="C80" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17860,10 +18487,10 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="28" t="str">
-        <x:v>Other biomass</x:v>
+        <x:v>Other liquid biofuels</x:v>
       </x:c>
       <x:c r="B81" s="28" t="str">
-        <x:v>15.03 Charcoal</x:v>
+        <x:v>16.08 Other liquid biofuels</x:v>
       </x:c>
       <x:c r="C81" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17871,10 +18498,10 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="28" t="str">
-        <x:v>Other biomass</x:v>
+        <x:v>Other products</x:v>
       </x:c>
       <x:c r="B82" s="28" t="str">
-        <x:v>15.05 Other biomass</x:v>
+        <x:v>07.17 Other products</x:v>
       </x:c>
       <x:c r="C82" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17882,21 +18509,21 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="28" t="str">
-        <x:v>Other bituminous coal</x:v>
+        <x:v>Other products</x:v>
       </x:c>
       <x:c r="B83" s="28" t="str">
-        <x:v>01.02 Other bituminous coal</x:v>
+        <x:v>07.17 Other products</x:v>
       </x:c>
       <x:c r="C83" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="28" t="str">
-        <x:v>Other hydrocarbons</x:v>
+        <x:v>Other recovered gases</x:v>
       </x:c>
       <x:c r="B84" s="28" t="str">
-        <x:v>06.05 Other hydrocarbons</x:v>
+        <x:v>02.05 Other recovered gases</x:v>
       </x:c>
       <x:c r="C84" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17904,21 +18531,21 @@
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="28" t="str">
-        <x:v>Other liquid biofuels</x:v>
+        <x:v>Other recovered gases</x:v>
       </x:c>
       <x:c r="B85" s="28" t="str">
-        <x:v>16.08 Other liquid biofuels</x:v>
+        <x:v>02.05 Other recovered gases</x:v>
       </x:c>
       <x:c r="C85" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="28" t="str">
-        <x:v>Other products</x:v>
+        <x:v>Other sources</x:v>
       </x:c>
       <x:c r="B86" s="28" t="str">
-        <x:v>07.17 Other products</x:v>
+        <x:v>16.09 Other sources</x:v>
       </x:c>
       <x:c r="C86" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17926,10 +18553,10 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="28" t="str">
-        <x:v>Other recovered gases</x:v>
+        <x:v>Paraffin waxes</x:v>
       </x:c>
       <x:c r="B87" s="28" t="str">
-        <x:v>02.04 Blast furnace gas</x:v>
+        <x:v>07.15 Paraffin waxes</x:v>
       </x:c>
       <x:c r="C87" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17937,10 +18564,10 @@
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="28" t="str">
-        <x:v>Other recovered gases</x:v>
+        <x:v>Patent fuel</x:v>
       </x:c>
       <x:c r="B88" s="28" t="str">
-        <x:v>02.05 Other recovered gases</x:v>
+        <x:v>02.06 Patent fuel</x:v>
       </x:c>
       <x:c r="C88" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17948,10 +18575,10 @@
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="28" t="str">
-        <x:v>Other sources</x:v>
+        <x:v>Peat</x:v>
       </x:c>
       <x:c r="B89" s="28" t="str">
-        <x:v>16.09 Other sources</x:v>
+        <x:v>03 Peat</x:v>
       </x:c>
       <x:c r="C89" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17959,10 +18586,10 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="28" t="str">
-        <x:v>Paraffin waxes</x:v>
+        <x:v>Peat products</x:v>
       </x:c>
       <x:c r="B90" s="28" t="str">
-        <x:v>07.15 Paraffin waxes</x:v>
+        <x:v>04 Peat products</x:v>
       </x:c>
       <x:c r="C90" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17970,10 +18597,10 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="28" t="str">
-        <x:v>Patent fuel</x:v>
+        <x:v>PetProd nonspecified</x:v>
       </x:c>
       <x:c r="B91" s="28" t="str">
-        <x:v>02.05 Other recovered gases</x:v>
+        <x:v>07.99 PetProd nonspecified</x:v>
       </x:c>
       <x:c r="C91" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17981,10 +18608,10 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="28" t="str">
-        <x:v>Patent fuel</x:v>
+        <x:v>Petroleum coke</x:v>
       </x:c>
       <x:c r="B92" s="28" t="str">
-        <x:v>02.06 Patent fuel</x:v>
+        <x:v>07.16 Petroleum coke</x:v>
       </x:c>
       <x:c r="C92" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -17992,21 +18619,21 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="28" t="str">
-        <x:v>Peat</x:v>
+        <x:v>Petroleum coke</x:v>
       </x:c>
       <x:c r="B93" s="28" t="str">
-        <x:v>03 Peat</x:v>
+        <x:v>07.16 Petroleum coke</x:v>
       </x:c>
       <x:c r="C93" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="28" t="str">
-        <x:v>Peat</x:v>
+        <x:v>Refinery feedstocks</x:v>
       </x:c>
       <x:c r="B94" s="28" t="str">
-        <x:v>18 Heat</x:v>
+        <x:v>06.03 Refinery feedstocks</x:v>
       </x:c>
       <x:c r="C94" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -18014,10 +18641,10 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="28" t="str">
-        <x:v>Peat products</x:v>
+        <x:v>Refinery gas not liquefied</x:v>
       </x:c>
       <x:c r="B95" s="28" t="str">
-        <x:v>03 Peat</x:v>
+        <x:v>07.10 Refinery gas (not liquefied)</x:v>
       </x:c>
       <x:c r="C95" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -18025,21 +18652,21 @@
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="28" t="str">
-        <x:v>Peat products</x:v>
+        <x:v>Refinery gas not liquefied</x:v>
       </x:c>
       <x:c r="B96" s="28" t="str">
-        <x:v>04 Peat products</x:v>
+        <x:v>07.10 Refinery gas (not liquefied)</x:v>
       </x:c>
       <x:c r="C96" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="28" t="str">
-        <x:v>PetProd nonspecified</x:v>
+        <x:v>Solar nonspecified</x:v>
       </x:c>
       <x:c r="B97" s="28" t="str">
-        <x:v>07.99 PetProd nonspecified</x:v>
+        <x:v>12.99 Solar nonspecified</x:v>
       </x:c>
       <x:c r="C97" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -18047,10 +18674,10 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="28" t="str">
-        <x:v>Petroleum coke</x:v>
+        <x:v>Solar photovoltaics</x:v>
       </x:c>
       <x:c r="B98" s="28" t="str">
-        <x:v>07.16 Petroleum coke</x:v>
+        <x:v>12.01 of which: Photovoltaics</x:v>
       </x:c>
       <x:c r="C98" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -18058,10 +18685,10 @@
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="28" t="str">
-        <x:v>Refinery feedstocks</x:v>
+        <x:v>Sub bituminous coal</x:v>
       </x:c>
       <x:c r="B99" s="28" t="str">
-        <x:v>06.03 Refinery feedstocks</x:v>
+        <x:v>01.03 Sub-bituminous coal</x:v>
       </x:c>
       <x:c r="C99" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -18069,21 +18696,21 @@
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="28" t="str">
-        <x:v>Refinery gas not liquefied</x:v>
+        <x:v>Sub bituminous coal</x:v>
       </x:c>
       <x:c r="B100" s="28" t="str">
-        <x:v>07.10 Refinery gas (not liquefied)</x:v>
+        <x:v>01.03 Sub-bituminous coal</x:v>
       </x:c>
       <x:c r="C100" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="28" t="str">
-        <x:v>Solar nonspecified</x:v>
+        <x:v>Tide wave ocean</x:v>
       </x:c>
       <x:c r="B101" s="28" t="str">
-        <x:v>11 Geothermal</x:v>
+        <x:v>13 Tide, wave, ocean</x:v>
       </x:c>
       <x:c r="C101" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -18091,10 +18718,10 @@
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="28" t="str">
-        <x:v>Solar nonspecified</x:v>
+        <x:v>White spirit SBP</x:v>
       </x:c>
       <x:c r="B102" s="28" t="str">
-        <x:v>12.99 Solar nonspecified</x:v>
+        <x:v>07.12 White spirit SBP</x:v>
       </x:c>
       <x:c r="C102" s="28" t="str">
         <x:v>BOTH</x:v>
@@ -18102,73 +18729,29 @@
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="28" t="str">
-        <x:v>Solar photovoltaics</x:v>
+        <x:v>White spirit SBP</x:v>
       </x:c>
       <x:c r="B103" s="28" t="str">
-        <x:v>12.01 of which: Photovoltaics</x:v>
+        <x:v>07.12 White spirit SBP</x:v>
       </x:c>
       <x:c r="C103" s="28" t="str">
-        <x:v>BOTH</x:v>
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
-      <x:c r="A104" s="28" t="str">
-        <x:v>Sub bituminous coal</x:v>
-      </x:c>
-      <x:c r="B104" s="28" t="str">
-        <x:v>01.02 Other bituminous coal</x:v>
-      </x:c>
-      <x:c r="C104" s="28" t="str">
-        <x:v>BOTH</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="105">
-      <x:c r="A105" s="28" t="str">
-        <x:v>Sub bituminous coal</x:v>
-      </x:c>
-      <x:c r="B105" s="28" t="str">
-        <x:v>01.03 Sub-bituminous coal</x:v>
-      </x:c>
-      <x:c r="C105" s="28" t="str">
-        <x:v>BOTH</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="106">
-      <x:c r="A106" s="28" t="str">
-        <x:v>Tide wave ocean</x:v>
-      </x:c>
-      <x:c r="B106" s="28" t="str">
-        <x:v>13 Tide, wave, ocean</x:v>
-      </x:c>
-      <x:c r="C106" s="28" t="str">
-        <x:v>BOTH</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="107">
-      <x:c r="A107" s="28" t="str">
-        <x:v>White spirit SBP</x:v>
-      </x:c>
-      <x:c r="B107" s="28" t="str">
-        <x:v>07.12 White spirit SBP</x:v>
-      </x:c>
-      <x:c r="C107" s="28" t="str">
-        <x:v>BOTH</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108">
-      <x:c r="A108" s="29" t="str">
+      <x:c r="A104" s="29" t="str">
         <x:v>Wind</x:v>
       </x:c>
-      <x:c r="B108" s="29" t="str">
+      <x:c r="B104" s="29" t="str">
         <x:v>14 Wind</x:v>
       </x:c>
-      <x:c r="C108" s="29" t="str">
+      <x:c r="C104" s="29" t="str">
         <x:v>BOTH</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" allowBlank="0" showDropDown="0" sqref="C2:C108">
+    <x:dataValidation type="list" allowBlank="0" showDropDown="0" sqref="C2:C104">
       <x:formula1>"BOTH,ESTO,ESTO_EXTENDED"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -19066,82 +19649,82 @@
     </x:row>
     <x:row r="111">
       <x:c r="A111" s="28" t="str">
-        <x:v>Total Primary Supply</x:v>
+        <x:v>Statistical Differences</x:v>
       </x:c>
       <x:c r="B111" s="28" t="str">
-        <x:v>07_total_primary_energy_supply</x:v>
+        <x:v>11_statistical_discrepancy</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
       <x:c r="A112" s="28" t="str">
-        <x:v>Total final consumption</x:v>
+        <x:v>Stock Changes</x:v>
       </x:c>
       <x:c r="B112" s="28" t="str">
-        <x:v>12_total_final_consumption</x:v>
+        <x:v>06_stock_changes</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
       <x:c r="A113" s="28" t="str">
-        <x:v>Total final energy consumption</x:v>
+        <x:v>Total Primary Supply</x:v>
       </x:c>
       <x:c r="B113" s="28" t="str">
-        <x:v>13_total_final_energy_consumption</x:v>
+        <x:v>07_total_primary_energy_supply</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
       <x:c r="A114" s="28" t="str">
-        <x:v>Total transformation - no transfers</x:v>
+        <x:v>Total final consumption</x:v>
       </x:c>
       <x:c r="B114" s="28" t="str">
-        <x:v>09_total_transformation_sector</x:v>
+        <x:v>12_total_final_consumption</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
       <x:c r="A115" s="28" t="str">
-        <x:v>Transfers</x:v>
+        <x:v>Total final energy consumption</x:v>
       </x:c>
       <x:c r="B115" s="28" t="str">
-        <x:v>08_transfers</x:v>
+        <x:v>13_total_final_energy_consumption</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
       <x:c r="A116" s="28" t="str">
-        <x:v>Transmission and Distribution</x:v>
+        <x:v>Total transformation - no transfers</x:v>
       </x:c>
       <x:c r="B116" s="28" t="str">
-        <x:v>10_02_transmission_and_distribution_losses</x:v>
+        <x:v>09_total_transformation_sector</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
       <x:c r="A117" s="28" t="str">
-        <x:v>Transport</x:v>
+        <x:v>Transfers</x:v>
       </x:c>
       <x:c r="B117" s="28" t="str">
-        <x:v>15_transport_sector</x:v>
+        <x:v>08_transfers</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
       <x:c r="A118" s="28" t="str">
-        <x:v>Transport non road</x:v>
+        <x:v>Transmission and Distribution</x:v>
       </x:c>
       <x:c r="B118" s="28" t="str">
-        <x:v>15_01,15_03-15_06 Transport non-road</x:v>
+        <x:v>10_02_transmission_and_distribution_losses</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" s="28" t="str">
-        <x:v>Transport non road/Freight non road</x:v>
+        <x:v>Transport</x:v>
       </x:c>
       <x:c r="B119" s="28" t="str">
-        <x:v>15_01_02_freight</x:v>
+        <x:v>15_transport_sector</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
       <x:c r="A120" s="28" t="str">
-        <x:v>Transport non road/Freight non road</x:v>
+        <x:v>Transport non road</x:v>
       </x:c>
       <x:c r="B120" s="28" t="str">
-        <x:v>15_03_02_freight</x:v>
+        <x:v>15_01,15_03-15_06 Transport non-road</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -19149,63 +19732,63 @@
         <x:v>Transport non road/Freight non road</x:v>
       </x:c>
       <x:c r="B121" s="28" t="str">
-        <x:v>15_04_02_freight</x:v>
+        <x:v>15_01_02_freight</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
       <x:c r="A122" s="28" t="str">
-        <x:v>Transport non road/Freight non road/Air</x:v>
+        <x:v>Transport non road/Freight non road</x:v>
       </x:c>
       <x:c r="B122" s="28" t="str">
-        <x:v>15_01_domestic_air_transport</x:v>
+        <x:v>15_03_02_freight</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
       <x:c r="A123" s="28" t="str">
-        <x:v>Transport non road/Freight non road/Rail</x:v>
+        <x:v>Transport non road/Freight non road</x:v>
       </x:c>
       <x:c r="B123" s="28" t="str">
-        <x:v>15_03_rail</x:v>
+        <x:v>15_04_02_freight</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="28" t="str">
-        <x:v>Transport non road/Freight non road/Shipping</x:v>
+        <x:v>Transport non road/Freight non road/Air</x:v>
       </x:c>
       <x:c r="B124" s="28" t="str">
-        <x:v>15_04_domestic_navigation</x:v>
+        <x:v>15_01_domestic_air_transport</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="28" t="str">
-        <x:v>Transport non road/International transport/Air</x:v>
+        <x:v>Transport non road/Freight non road/Rail</x:v>
       </x:c>
       <x:c r="B125" s="28" t="str">
-        <x:v>05_international_aviation_bunkers</x:v>
+        <x:v>15_03_rail</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="28" t="str">
-        <x:v>Transport non road/International transport/Shipping</x:v>
+        <x:v>Transport non road/Freight non road/Shipping</x:v>
       </x:c>
       <x:c r="B126" s="28" t="str">
-        <x:v>04_international_marine_bunkers</x:v>
+        <x:v>15_04_domestic_navigation</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="28" t="str">
-        <x:v>Transport non road/Nonspecified transport</x:v>
+        <x:v>Transport non road/International transport/Air</x:v>
       </x:c>
       <x:c r="B127" s="28" t="str">
-        <x:v>15_02_road</x:v>
+        <x:v>05_international_aviation_bunkers</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="28" t="str">
-        <x:v>Transport non road/Nonspecified transport</x:v>
+        <x:v>Transport non road/International transport/Shipping</x:v>
       </x:c>
       <x:c r="B128" s="28" t="str">
-        <x:v>15_03_rail</x:v>
+        <x:v>04_international_marine_bunkers</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -19213,23 +19796,23 @@
         <x:v>Transport non road/Nonspecified transport</x:v>
       </x:c>
       <x:c r="B129" s="28" t="str">
-        <x:v>15_06_nonspecified_transport</x:v>
+        <x:v>15_02_road</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="28" t="str">
-        <x:v>Transport non road/Passenger non road</x:v>
+        <x:v>Transport non road/Nonspecified transport</x:v>
       </x:c>
       <x:c r="B130" s="28" t="str">
-        <x:v>15_01_01_passenger</x:v>
+        <x:v>15_03_rail</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="28" t="str">
-        <x:v>Transport non road/Passenger non road</x:v>
+        <x:v>Transport non road/Nonspecified transport</x:v>
       </x:c>
       <x:c r="B131" s="28" t="str">
-        <x:v>15_03_01_passenger</x:v>
+        <x:v>15_06_nonspecified_transport</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -19237,38 +19820,54 @@
         <x:v>Transport non road/Passenger non road</x:v>
       </x:c>
       <x:c r="B132" s="28" t="str">
-        <x:v>15_04_01_passenger</x:v>
+        <x:v>15_01_01_passenger</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="28" t="str">
-        <x:v>Transport non road/Passenger non road/Air</x:v>
+        <x:v>Transport non road/Passenger non road</x:v>
       </x:c>
       <x:c r="B133" s="28" t="str">
-        <x:v>15_01_domestic_air_transport</x:v>
+        <x:v>15_03_01_passenger</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="28" t="str">
-        <x:v>Transport non road/Passenger non road/Rail</x:v>
+        <x:v>Transport non road/Passenger non road</x:v>
       </x:c>
       <x:c r="B134" s="28" t="str">
-        <x:v>15_03_rail</x:v>
+        <x:v>15_04_01_passenger</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="28" t="str">
+        <x:v>Transport non road/Passenger non road/Air</x:v>
+      </x:c>
+      <x:c r="B135" s="28" t="str">
+        <x:v>15_01_domestic_air_transport</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="28" t="str">
+        <x:v>Transport non road/Passenger non road/Rail</x:v>
+      </x:c>
+      <x:c r="B136" s="28" t="str">
+        <x:v>15_03_rail</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="28" t="str">
         <x:v>Transport non road/Passenger non road/Shipping</x:v>
       </x:c>
-      <x:c r="B135" s="28" t="str">
+      <x:c r="B137" s="28" t="str">
         <x:v>15_04_domestic_navigation</x:v>
       </x:c>
     </x:row>
-    <x:row r="136">
-      <x:c r="A136" s="29" t="str">
+    <x:row r="138">
+      <x:c r="A138" s="29" t="str">
         <x:v>Transport non road/Pipeline transport</x:v>
       </x:c>
-      <x:c r="B136" s="29" t="str">
+      <x:c r="B138" s="29" t="str">
         <x:v>15_05_pipeline_transport</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
codex: remove duplicate editable axis mappings
Deduplicate normalized mapping keys across all ten editable sheets during every separate-axis refresh, preserve distinct targets, and record a per-sheet cleanup audit. Refresh the user-facing workbook README and regenerate the production mapping workbooks.\n\nVerification: injected-duplicate workbook integration test passed; final editable workbook has zero duplicates and zero formula errors; 77 focused mapping tests passed; production separate-axis refresh promoted successfully.
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd5a04c2b4a784b9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="Raf517561891449c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R5f4ce45fe51d4f3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R15a9de2067344e8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R5add99920203428c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Rfe7ad548d9c949e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="R5f9279f3c8f74b3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Rc83eeef31c014233"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="Rd4c7fe93fc0849c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R2712722cdb164887"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R211d1f1de7b74de8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7547607b34214f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R0505d7c55e994ac0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R5b69ff03e4c94f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R33f10cfb2bea4cae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="Rd326ea66578946db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R0065b3792e314a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rc49992e9cbc8496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Re3ba776f9592445b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R2f0e83fb0e9d4cab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R9838e4f6799b4e1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R1661cba4ec434a82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -505,7 +505,7 @@
         <x:v>Allowed cardinality</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>One-to-one, one-to-many, and many-to-one relationships are supported. A many-to-many connected component within one axis is blocking QA and must be reviewed.</x:v>
+        <x:v>One-to-one, one-to-many, and many-to-one relationships are supported. Small many-to-many components remain review items; oversized or cross-family product components block compilation.</x:v>
       </x:c>
       <x:c r="C8" s="19"/>
       <x:c r="D8" s="19"/>
@@ -558,10 +558,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="16" t="str">
-        <x:v>Subtotals and rollups</x:v>
+        <x:v>Duplicate rows</x:v>
       </x:c>
       <x:c r="B12" s="17" t="str">
-        <x:v>Canonical rollup rules are applied to raw key pairs before mappings are compiled. The generated master keeps the existing rollup-rule sheets unchanged.</x:v>
+        <x:v>Each refresh keeps the first occurrence of an exact mapping key and removes later duplicates from this workbook. Different targets remain valid one-to-many mappings.</x:v>
       </x:c>
       <x:c r="C12" s="19"/>
       <x:c r="D12" s="19"/>
@@ -572,10 +572,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="16" t="str">
-        <x:v>Current status</x:v>
+        <x:v>Subtotals and rollups</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>Production contract with explicit semantic review debt.</x:v>
+        <x:v>Canonical rollup rules are applied to raw key pairs before mappings are compiled. The generated master keeps the existing rollup-rule sheets unchanged.</x:v>
       </x:c>
       <x:c r="C13" s="19"/>
       <x:c r="D13" s="19"/>
@@ -585,8 +585,12 @@
       <x:c r="H13" s="19"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="19"/>
-      <x:c r="B14" s="19"/>
+      <x:c r="A14" s="16" t="str">
+        <x:v>Current status</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str">
+        <x:v>Production contract with explicit semantic review debt.</x:v>
+      </x:c>
       <x:c r="C14" s="19"/>
       <x:c r="D14" s="19"/>
       <x:c r="E14" s="19"/>

</xml_diff>

<commit_message>
codex: map green electricity to hydrogen fuel
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R600b4703b2594f66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="Re1b300d4008840c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R49688c5700e54aa3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="Re2ceb73a3d864495"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R532ca50aaa8249a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Re0de785e12ee4e64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="R5bdeadd79c7843a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="R551dc3b4b38a412d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R845b5dab171a4024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R138a6665b2514462"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R32e65ab80c384bc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R2711ebf8a9b74da8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="R7cce226b34634cc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Rcee185841ce44d83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R3334093862c34718"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="R5f3e10ca4ed7486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra18db23425204207"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R39e32e6b775a40a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R5099b1ebe6e949ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="Rdfeafdf190ee4867"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R554b81c32977405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Rb094f630d6944584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rf80c45dc190d482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="R65a65bd7b7e24089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R2292041ab3c34050"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="Rc0666bfd88134209"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="Rc951c64eab254969"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R3d8e70775b5f422c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="Rb5915baf5d0545b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="R5145193288d84892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R1af8921b2d4c4a1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="R25fda17cd39e44a7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -354,13 +354,13 @@
     <xdr:ext cx="11239500" cy="2238375"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="/xl/media/image1.png"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra095c7c8214b4333"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1168d1ec7b724c09"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1023,7 +1023,7 @@
     <x:mergeCell ref="A4:H4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R319ead4fe87e4c14"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79b490924aa54257"/>
 </x:worksheet>
 </file>
 
@@ -36233,10 +36233,8 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="37" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Electricity</x:t>
-        </x:is>
+      <x:c r="A24" s="37" t="str">
+        <x:v>Electricity for hydrogen</x:v>
       </x:c>
       <x:c r="B24" s="37" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
codex: align LEAP TPES rollup boundary
Verification: python -m pytest -q tests/test_source_rollups.py tests/test_tpes_rollup_configuration.py tests/test_tfc_rollup_configuration.py (9 passed).
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfc6d3a784cea4812"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R1c73f5dbf17a4fa0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R6d49557a60184923"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R400118f7644a4f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R1b7d1188174649d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Rc3e457ecd19a465a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="R6313eb87c3b04bc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Rf8bc38c32a2d4146"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="Redc72d8c30e346e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="Rcab4a18687364403"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="Re1080b2a182147eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R2ab98da6caf24460"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="Rf085bdc86a324c24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Rd07f33d87e43437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R8c167a2128ec4ba7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="Rb72d7145f2ed4e6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R943188c2548046a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R5485c94171654f7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R81a9a8c49b434739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R4f040bb522644d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="Rada44de1dd0c4e0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R0b9105b6e6b54393"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Reeeeb9e3eda04cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="R9a4997f7c2274915"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R037b821e92864cd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="Rac03d217b2f443d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R8db7026276f1442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R735c01d516634f8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="Re2830cc9147d45f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Ra27fe0a0ed504fa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="Rd19cb520ecb645e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="R2ed7e9a952ab442e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -152,7 +152,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="45">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0"/>
@@ -262,6 +262,21 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyAlignment="1">
+      <x:alignment vertical="top"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -355,7 +370,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re6cff60e037644ad"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R77fc8060515345b1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1018,7 +1033,7 @@
     <x:mergeCell ref="A4:H4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8137cf435c144856"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e10dc024a45488b"/>
 </x:worksheet>
 </file>
 
@@ -19972,6 +19987,9 @@
       <x:c r="N1" s="25" t="str">
         <x:v>priority</x:v>
       </x:c>
+      <x:c r="O1" t="str">
+        <x:v>input_value_multiplier</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="39" t="str">
@@ -20004,6 +20022,9 @@
       <x:c r="L2" s="39"/>
       <x:c r="M2" s="39"/>
       <x:c r="N2" s="39"/>
+      <x:c r="O2" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="40" t="str">
@@ -20036,6 +20057,9 @@
       <x:c r="L3" s="40"/>
       <x:c r="M3" s="40"/>
       <x:c r="N3" s="40"/>
+      <x:c r="O3" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="40" t="str">
@@ -20068,6 +20092,9 @@
       <x:c r="L4" s="40"/>
       <x:c r="M4" s="40"/>
       <x:c r="N4" s="40"/>
+      <x:c r="O4" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="40" t="str">
@@ -20100,6 +20127,9 @@
       <x:c r="L5" s="40"/>
       <x:c r="M5" s="40"/>
       <x:c r="N5" s="40"/>
+      <x:c r="O5" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="40" t="str">
@@ -20132,6 +20162,9 @@
       <x:c r="L6" s="40"/>
       <x:c r="M6" s="40"/>
       <x:c r="N6" s="40"/>
+      <x:c r="O6" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="40" t="str">
@@ -20164,6 +20197,9 @@
       <x:c r="L7" s="40"/>
       <x:c r="M7" s="40"/>
       <x:c r="N7" s="40"/>
+      <x:c r="O7" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="40" t="str">
@@ -20196,6 +20232,9 @@
       <x:c r="L8" s="40"/>
       <x:c r="M8" s="40"/>
       <x:c r="N8" s="40"/>
+      <x:c r="O8" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="40" t="str">
@@ -20228,6 +20267,9 @@
       <x:c r="L9" s="40"/>
       <x:c r="M9" s="40"/>
       <x:c r="N9" s="40"/>
+      <x:c r="O9" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="40" t="str">
@@ -20260,6 +20302,9 @@
       <x:c r="L10" s="40"/>
       <x:c r="M10" s="40"/>
       <x:c r="N10" s="40"/>
+      <x:c r="O10" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="40" t="str">
@@ -20292,6 +20337,9 @@
       <x:c r="L11" s="40"/>
       <x:c r="M11" s="40"/>
       <x:c r="N11" s="40"/>
+      <x:c r="O11" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="40" t="str">
@@ -20322,6 +20370,9 @@
       <x:c r="L12" s="40"/>
       <x:c r="M12" s="40"/>
       <x:c r="N12" s="40"/>
+      <x:c r="O12" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="40" t="str">
@@ -20352,6 +20403,9 @@
       <x:c r="L13" s="40"/>
       <x:c r="M13" s="40"/>
       <x:c r="N13" s="40"/>
+      <x:c r="O13" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="40" t="str">
@@ -20382,6 +20436,9 @@
       <x:c r="L14" s="40"/>
       <x:c r="M14" s="40"/>
       <x:c r="N14" s="40"/>
+      <x:c r="O14" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="40" t="str">
@@ -20414,6 +20471,9 @@
       <x:c r="L15" s="40"/>
       <x:c r="M15" s="40"/>
       <x:c r="N15" s="40"/>
+      <x:c r="O15" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="40" t="str">
@@ -20446,6 +20506,9 @@
       <x:c r="L16" s="40"/>
       <x:c r="M16" s="40"/>
       <x:c r="N16" s="40"/>
+      <x:c r="O16" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="40" t="str">
@@ -20478,6 +20541,9 @@
       <x:c r="L17" s="40"/>
       <x:c r="M17" s="40"/>
       <x:c r="N17" s="40"/>
+      <x:c r="O17" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="40" t="str">
@@ -20510,6 +20576,9 @@
       <x:c r="L18" s="40"/>
       <x:c r="M18" s="40"/>
       <x:c r="N18" s="40"/>
+      <x:c r="O18" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="40" t="str">
@@ -20542,6 +20611,9 @@
       <x:c r="L19" s="40"/>
       <x:c r="M19" s="40"/>
       <x:c r="N19" s="40"/>
+      <x:c r="O19" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="40" t="str">
@@ -20574,6 +20646,9 @@
       <x:c r="L20" s="40"/>
       <x:c r="M20" s="40"/>
       <x:c r="N20" s="40"/>
+      <x:c r="O20" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="40" t="str">
@@ -20606,6 +20681,9 @@
       <x:c r="L21" s="40"/>
       <x:c r="M21" s="40"/>
       <x:c r="N21" s="40"/>
+      <x:c r="O21" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="40" t="str">
@@ -20638,6 +20716,9 @@
       <x:c r="L22" s="40"/>
       <x:c r="M22" s="40"/>
       <x:c r="N22" s="40"/>
+      <x:c r="O22" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="40" t="str">
@@ -20670,6 +20751,9 @@
       <x:c r="L23" s="40"/>
       <x:c r="M23" s="40"/>
       <x:c r="N23" s="40"/>
+      <x:c r="O23" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="40" t="str">
@@ -20702,6 +20786,9 @@
       <x:c r="L24" s="40"/>
       <x:c r="M24" s="40"/>
       <x:c r="N24" s="40"/>
+      <x:c r="O24" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="40" t="str">
@@ -20734,6 +20821,9 @@
       <x:c r="L25" s="40"/>
       <x:c r="M25" s="40"/>
       <x:c r="N25" s="40"/>
+      <x:c r="O25" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="40" t="str">
@@ -20766,6 +20856,9 @@
       <x:c r="L26" s="40"/>
       <x:c r="M26" s="40"/>
       <x:c r="N26" s="40"/>
+      <x:c r="O26" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="40" t="str">
@@ -20796,6 +20889,9 @@
       <x:c r="L27" s="40"/>
       <x:c r="M27" s="40"/>
       <x:c r="N27" s="40"/>
+      <x:c r="O27" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="40" t="str">
@@ -20826,6 +20922,9 @@
       <x:c r="L28" s="40"/>
       <x:c r="M28" s="40"/>
       <x:c r="N28" s="40"/>
+      <x:c r="O28" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="40" t="str">
@@ -20856,6 +20955,9 @@
       <x:c r="L29" s="40"/>
       <x:c r="M29" s="40"/>
       <x:c r="N29" s="40"/>
+      <x:c r="O29" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="40" t="str">
@@ -20886,6 +20988,9 @@
       <x:c r="L30" s="40"/>
       <x:c r="M30" s="40"/>
       <x:c r="N30" s="40"/>
+      <x:c r="O30" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="40" t="str">
@@ -20916,6 +21021,9 @@
       <x:c r="L31" s="40"/>
       <x:c r="M31" s="40"/>
       <x:c r="N31" s="40"/>
+      <x:c r="O31" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="40" t="str">
@@ -20946,6 +21054,9 @@
       <x:c r="L32" s="40"/>
       <x:c r="M32" s="40"/>
       <x:c r="N32" s="40"/>
+      <x:c r="O32" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="40" t="str">
@@ -20976,6 +21087,9 @@
       <x:c r="L33" s="40"/>
       <x:c r="M33" s="40"/>
       <x:c r="N33" s="40"/>
+      <x:c r="O33" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="40" t="str">
@@ -21006,6 +21120,9 @@
       <x:c r="L34" s="40"/>
       <x:c r="M34" s="40"/>
       <x:c r="N34" s="40"/>
+      <x:c r="O34" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="40" t="str">
@@ -21036,6 +21153,9 @@
       <x:c r="L35" s="40"/>
       <x:c r="M35" s="40"/>
       <x:c r="N35" s="40"/>
+      <x:c r="O35" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="40" t="str">
@@ -21066,6 +21186,9 @@
       <x:c r="L36" s="40"/>
       <x:c r="M36" s="40"/>
       <x:c r="N36" s="40"/>
+      <x:c r="O36" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="40" t="str">
@@ -21096,6 +21219,9 @@
       <x:c r="L37" s="40"/>
       <x:c r="M37" s="40"/>
       <x:c r="N37" s="40"/>
+      <x:c r="O37" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="40" t="str">
@@ -21126,6 +21252,9 @@
       <x:c r="L38" s="40"/>
       <x:c r="M38" s="40"/>
       <x:c r="N38" s="40"/>
+      <x:c r="O38" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="40" t="str">
@@ -21156,6 +21285,9 @@
       <x:c r="L39" s="40"/>
       <x:c r="M39" s="40"/>
       <x:c r="N39" s="40"/>
+      <x:c r="O39" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="40" t="str">
@@ -21186,6 +21318,9 @@
       <x:c r="L40" s="40"/>
       <x:c r="M40" s="40"/>
       <x:c r="N40" s="40"/>
+      <x:c r="O40" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="40" t="str">
@@ -21216,6 +21351,9 @@
       <x:c r="L41" s="40"/>
       <x:c r="M41" s="40"/>
       <x:c r="N41" s="40"/>
+      <x:c r="O41" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="40" t="str">
@@ -21246,6 +21384,9 @@
       <x:c r="L42" s="40"/>
       <x:c r="M42" s="40"/>
       <x:c r="N42" s="40"/>
+      <x:c r="O42" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="40" t="str">
@@ -21276,6 +21417,9 @@
       <x:c r="L43" s="40"/>
       <x:c r="M43" s="40"/>
       <x:c r="N43" s="40"/>
+      <x:c r="O43" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="40" t="str">
@@ -21306,6 +21450,9 @@
       <x:c r="L44" s="40"/>
       <x:c r="M44" s="40"/>
       <x:c r="N44" s="40"/>
+      <x:c r="O44" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="40" t="str">
@@ -21336,6 +21483,9 @@
       <x:c r="L45" s="40"/>
       <x:c r="M45" s="40"/>
       <x:c r="N45" s="40"/>
+      <x:c r="O45" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="40" t="str">
@@ -21366,6 +21516,9 @@
       <x:c r="L46" s="40"/>
       <x:c r="M46" s="40"/>
       <x:c r="N46" s="40"/>
+      <x:c r="O46" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="40" t="str">
@@ -21396,6 +21549,9 @@
       <x:c r="L47" s="40"/>
       <x:c r="M47" s="40"/>
       <x:c r="N47" s="40"/>
+      <x:c r="O47" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="40" t="str">
@@ -21426,6 +21582,9 @@
       <x:c r="L48" s="40"/>
       <x:c r="M48" s="40"/>
       <x:c r="N48" s="40"/>
+      <x:c r="O48" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="40" t="str">
@@ -21456,6 +21615,9 @@
       <x:c r="L49" s="40"/>
       <x:c r="M49" s="40"/>
       <x:c r="N49" s="40"/>
+      <x:c r="O49" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="40" t="str">
@@ -21486,6 +21648,9 @@
       <x:c r="L50" s="40"/>
       <x:c r="M50" s="40"/>
       <x:c r="N50" s="40"/>
+      <x:c r="O50" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="40" t="str">
@@ -21516,6 +21681,9 @@
       <x:c r="L51" s="40"/>
       <x:c r="M51" s="40"/>
       <x:c r="N51" s="40"/>
+      <x:c r="O51" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="40" t="str">
@@ -21546,6 +21714,9 @@
       <x:c r="L52" s="40"/>
       <x:c r="M52" s="40"/>
       <x:c r="N52" s="40"/>
+      <x:c r="O52" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="40" t="str">
@@ -21576,6 +21747,9 @@
       <x:c r="L53" s="40"/>
       <x:c r="M53" s="40"/>
       <x:c r="N53" s="40"/>
+      <x:c r="O53" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="40" t="str">
@@ -21606,6 +21780,9 @@
       <x:c r="L54" s="40"/>
       <x:c r="M54" s="40"/>
       <x:c r="N54" s="40"/>
+      <x:c r="O54" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="40" t="str">
@@ -21636,6 +21813,9 @@
       <x:c r="L55" s="40"/>
       <x:c r="M55" s="40"/>
       <x:c r="N55" s="40"/>
+      <x:c r="O55" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="40" t="str">
@@ -21666,6 +21846,9 @@
       <x:c r="L56" s="40"/>
       <x:c r="M56" s="40"/>
       <x:c r="N56" s="40"/>
+      <x:c r="O56" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="40" t="str">
@@ -21696,6 +21879,9 @@
       <x:c r="L57" s="40"/>
       <x:c r="M57" s="40"/>
       <x:c r="N57" s="40"/>
+      <x:c r="O57" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="40" t="str">
@@ -21726,6 +21912,9 @@
       <x:c r="L58" s="40"/>
       <x:c r="M58" s="40"/>
       <x:c r="N58" s="40"/>
+      <x:c r="O58" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="40" t="str">
@@ -21756,6 +21945,9 @@
       <x:c r="L59" s="40"/>
       <x:c r="M59" s="40"/>
       <x:c r="N59" s="40"/>
+      <x:c r="O59" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="40" t="str">
@@ -21786,6 +21978,9 @@
       <x:c r="L60" s="40"/>
       <x:c r="M60" s="40"/>
       <x:c r="N60" s="40"/>
+      <x:c r="O60" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="40" t="str">
@@ -21816,6 +22011,9 @@
       <x:c r="L61" s="40"/>
       <x:c r="M61" s="40"/>
       <x:c r="N61" s="40"/>
+      <x:c r="O61" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="40" t="str">
@@ -21848,6 +22046,9 @@
       <x:c r="L62" s="40"/>
       <x:c r="M62" s="40"/>
       <x:c r="N62" s="40"/>
+      <x:c r="O62" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="40" t="str">
@@ -21880,6 +22081,9 @@
       <x:c r="L63" s="40"/>
       <x:c r="M63" s="40"/>
       <x:c r="N63" s="40"/>
+      <x:c r="O63" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="40" t="str">
@@ -21912,6 +22116,9 @@
       <x:c r="L64" s="40"/>
       <x:c r="M64" s="40"/>
       <x:c r="N64" s="40"/>
+      <x:c r="O64" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="40" t="str">
@@ -21944,6 +22151,9 @@
       <x:c r="L65" s="40"/>
       <x:c r="M65" s="40"/>
       <x:c r="N65" s="40"/>
+      <x:c r="O65" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="40" t="str">
@@ -21976,6 +22186,9 @@
       <x:c r="L66" s="40"/>
       <x:c r="M66" s="40"/>
       <x:c r="N66" s="40"/>
+      <x:c r="O66" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="40" t="str">
@@ -22008,6 +22221,9 @@
       <x:c r="L67" s="40"/>
       <x:c r="M67" s="40"/>
       <x:c r="N67" s="40"/>
+      <x:c r="O67" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="40" t="str">
@@ -22038,31 +22254,132 @@
       <x:c r="L68" s="40"/>
       <x:c r="M68" s="40"/>
       <x:c r="N68" s="40"/>
+      <x:c r="O68" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="69">
-      <x:c r="A69" s="41"/>
-      <x:c r="B69" s="41"/>
-      <x:c r="C69" s="41"/>
-      <x:c r="D69" s="41"/>
-      <x:c r="E69" s="41"/>
-      <x:c r="F69" s="41"/>
-      <x:c r="G69" s="41"/>
-      <x:c r="H69" s="41"/>
-      <x:c r="I69" s="41"/>
-      <x:c r="J69" s="41"/>
-      <x:c r="K69" s="41"/>
-      <x:c r="L69" s="41"/>
-      <x:c r="M69" s="41"/>
-      <x:c r="N69" s="41"/>
+      <x:c r="A69" s="41" t="str">
+        <x:v>Total Primary Supply</x:v>
+      </x:c>
+      <x:c r="B69" s="41" t="str"/>
+      <x:c r="C69" s="41" t="str">
+        <x:v>Total Primary Supply including international transport adjustment</x:v>
+      </x:c>
+      <x:c r="D69" s="41" t="str"/>
+      <x:c r="E69" s="41" t="str">
+        <x:v>NON_EXPANDING</x:v>
+      </x:c>
+      <x:c r="F69" s="45" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G69" s="41" t="str">
+        <x:v>Net TPES boundary: retain gross LEAP supply before subtracting international transport.</x:v>
+      </x:c>
+      <x:c r="H69" s="45" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I69" s="41" t="str"/>
+      <x:c r="J69" s="41" t="str">
+        <x:v>Total Primary Supply; All demand aggregated/International transport</x:v>
+      </x:c>
+      <x:c r="K69" s="41" t="str">
+        <x:v>supply_balance</x:v>
+      </x:c>
+      <x:c r="L69" s="41" t="str">
+        <x:v>leap_tpes_net_bunkers</x:v>
+      </x:c>
+      <x:c r="M69" s="41" t="str">
+        <x:v>International transport is removed from domestic primary supply.</x:v>
+      </x:c>
+      <x:c r="N69" s="41" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O69" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="70">
-      <x:c r="A70"/>
-      <x:c r="C70"/>
-      <x:c r="E70"/>
-      <x:c r="F70"/>
-      <x:c r="G70"/>
-      <x:c r="H70"/>
-      <x:c r="J70"/>
+      <x:c r="A70" t="str">
+        <x:v>All demand aggregated/International transport</x:v>
+      </x:c>
+      <x:c r="B70" t="str"/>
+      <x:c r="C70" t="str">
+        <x:v>Total Primary Supply including international transport adjustment</x:v>
+      </x:c>
+      <x:c r="D70" t="str"/>
+      <x:c r="E70" t="str">
+        <x:v>NON_EXPANDING</x:v>
+      </x:c>
+      <x:c r="F70" s="46" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>Net TPES boundary: subtract the positive LEAP international-transport placeholder.</x:v>
+      </x:c>
+      <x:c r="H70" s="46" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I70" t="str"/>
+      <x:c r="J70" t="str">
+        <x:v>Total Primary Supply; All demand aggregated/International transport</x:v>
+      </x:c>
+      <x:c r="K70" t="str">
+        <x:v>supply_balance</x:v>
+      </x:c>
+      <x:c r="L70" t="str">
+        <x:v>leap_tpes_net_bunkers</x:v>
+      </x:c>
+      <x:c r="M70" t="str">
+        <x:v>International transport is removed from domestic primary supply.</x:v>
+      </x:c>
+      <x:c r="N70" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O70" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>All demand aggregated/International transport</x:v>
+      </x:c>
+      <x:c r="B71" t="str"/>
+      <x:c r="C71" t="str">
+        <x:v>International transport signed for supply</x:v>
+      </x:c>
+      <x:c r="D71" t="str"/>
+      <x:c r="E71" t="str">
+        <x:v>NON_EXPANDING</x:v>
+      </x:c>
+      <x:c r="F71" s="46" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>Publish the positive LEAP placeholder on the ESTO bunker axis with the balance-table negative sign.</x:v>
+      </x:c>
+      <x:c r="H71" s="46" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I71" t="str"/>
+      <x:c r="J71" t="str">
+        <x:v>All demand aggregated/International transport</x:v>
+      </x:c>
+      <x:c r="K71" t="str">
+        <x:v>supply_balance</x:v>
+      </x:c>
+      <x:c r="L71" t="str">
+        <x:v>leap_signed_international_transport</x:v>
+      </x:c>
+      <x:c r="M71" t="str">
+        <x:v>International transport is a supply deduction, not domestic demand.</x:v>
+      </x:c>
+      <x:c r="N71" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="O71" t="n">
+        <x:v>-1</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -26623,10 +26940,8 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">All demand aggregated/International transport</x:t>
-        </x:is>
+      <x:c r="A5" s="40" t="str">
+        <x:v>International transport signed for supply</x:v>
       </x:c>
       <x:c r="B5" s="40" t="inlineStr">
         <x:is>
@@ -28850,10 +29165,8 @@
       </x:c>
     </x:row>
     <x:row r="136">
-      <x:c r="A136" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Total Primary Supply</x:t>
-        </x:is>
+      <x:c r="A136" s="40" t="str">
+        <x:v>Total Primary Supply including international transport adjustment</x:v>
       </x:c>
       <x:c r="B136" s="40" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
codex: remove duplicate LEAP TFC rollups
Disable obsolete parent and legacy standalone TFC rollups so only the five domestic All demand aggregated child branches contribute. Regenerate canonical mapping workbooks and manifest.\n\nVerified: 48 focused mapping tests passed; Stage 3 completed; USA dashboard publish-readiness passed; 2028 LEAP Target TFC is 71,344.77 PJ versus Ninth 71,344.83 PJ.
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3d7673537e954ddc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R9996e29d7a8146d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R4c5ee525eeea4add"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R02cb0a6046984458"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R892a06166057420f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R319b09f7d2e84ca6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rc20b0dd265a44f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Rb2c3b99091264417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="Rc02770d8eaf64a46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R3f0472fdb5264aa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R918a5ca09d6e4d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="Rc671ab11b414489a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="R15accda837f3427f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Rbcdeeb7c2ca04d2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R3ff36c841e1742a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="Rf54a1b69248e40d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc173ae70fd284f2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R45c006f0dd7b4387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="Rab40633e59aa441f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R88accd8125754308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="Rcf2d80717c2e4836"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R3de4ee4bf1e74528"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rf10a5b9e284e4dbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Rc2d1c6f1acb94427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R71f047b540dd43d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="Rf917270686174d19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="Rbffc4d9d59144fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R5a0d3efcc43149fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="R00ab7bc776df451c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Rd462de5c740844a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R3075e9f4c7044606"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="R33c7c19ab0174359"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,7 +370,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6306f1b026a94835"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R375385ade1fc40dc"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1033,7 +1033,7 @@
     <x:mergeCell ref="A4:H4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb5644441b234081"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15bc2bb6e9a84f6b"/>
 </x:worksheet>
 </file>
 
@@ -22394,10 +22394,10 @@
         <x:v>NON_EXPANDING</x:v>
       </x:c>
       <x:c r="F72" s="46" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G72" t="str">
-        <x:v>Used for total final consumption comparison; should be kept separate from detailed demand-sector views to avoid double counting.</x:v>
+        <x:v>Disabled: superseded by the five domestic All demand aggregated child rollups; keeping this active double-counts TFC.</x:v>
       </x:c>
       <x:c r="H72" s="46" t="b">
         <x:v>1</x:v>
@@ -22425,10 +22425,10 @@
         <x:v>NON_EXPANDING</x:v>
       </x:c>
       <x:c r="F73" s="46" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G73" t="str">
-        <x:v>Used for total final consumption comparison; should be kept separate from detailed demand-sector views to avoid double counting.</x:v>
+        <x:v>Disabled: superseded by the five domestic All demand aggregated child rollups; keeping this active double-counts TFC.</x:v>
       </x:c>
       <x:c r="H73" s="46" t="b">
         <x:v>1</x:v>
@@ -22456,10 +22456,10 @@
         <x:v>NON_EXPANDING</x:v>
       </x:c>
       <x:c r="F74" s="46" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G74" t="str">
-        <x:v>Used for total final consumption comparison; should be kept separate from detailed demand-sector views to avoid double counting.</x:v>
+        <x:v>Disabled: superseded by the five domestic All demand aggregated child rollups; keeping this active double-counts TFC.</x:v>
       </x:c>
       <x:c r="H74" s="46" t="b">
         <x:v>1</x:v>
@@ -22487,10 +22487,10 @@
         <x:v>NON_EXPANDING</x:v>
       </x:c>
       <x:c r="F75" s="46" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G75" t="str">
-        <x:v>Used for total final consumption comparison; should be kept separate from detailed demand-sector views to avoid double counting.</x:v>
+        <x:v>Disabled: superseded by the five domestic All demand aggregated child rollups; keeping this active double-counts TFC.</x:v>
       </x:c>
       <x:c r="H75" s="46" t="b">
         <x:v>1</x:v>
@@ -22518,10 +22518,10 @@
         <x:v>NON_EXPANDING</x:v>
       </x:c>
       <x:c r="F76" s="46" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G76" t="str">
-        <x:v>Used for total final consumption comparison; should be kept separate from detailed demand-sector views to avoid double counting.</x:v>
+        <x:v>Disabled: superseded by the five domestic All demand aggregated child rollups; keeping this active double-counts TFC.</x:v>
       </x:c>
       <x:c r="H76" s="46" t="b">
         <x:v>1</x:v>
@@ -22549,10 +22549,10 @@
         <x:v>NON_EXPANDING</x:v>
       </x:c>
       <x:c r="F77" s="46" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G77" t="str">
-        <x:v>Used for total final consumption comparison; should be kept separate from detailed demand-sector views to avoid double counting.</x:v>
+        <x:v>Disabled: superseded by the five domestic All demand aggregated child rollups; keeping this active double-counts TFC.</x:v>
       </x:c>
       <x:c r="H77" s="46" t="b">
         <x:v>1</x:v>
@@ -22580,10 +22580,10 @@
         <x:v>NON_EXPANDING</x:v>
       </x:c>
       <x:c r="F78" s="46" t="b">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G78" t="str">
-        <x:v>Used for total final consumption comparison; should be kept separate from detailed demand-sector views to avoid double counting.</x:v>
+        <x:v>Disabled: superseded by the five domestic All demand aggregated child rollups; keeping this active double-counts TFC.</x:v>
       </x:c>
       <x:c r="H78" s="46" t="b">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
codex: restore coke and blast own-use boundaries
Activates the four NINTH leaf-level NON_EXPANDING rules in the single-axis authority and regenerated mapping workbooks. Verification: 42 focused mapping tests passed. Full pipeline output validation remains MAPQ-046's next gate.
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc173ae70fd284f2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R45c006f0dd7b4387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="Rab40633e59aa441f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R88accd8125754308"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="Rcf2d80717c2e4836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R3de4ee4bf1e74528"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rf10a5b9e284e4dbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Rc2d1c6f1acb94427"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R71f047b540dd43d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="Rf917270686174d19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="Rbffc4d9d59144fff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R5a0d3efcc43149fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="R00ab7bc776df451c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Rd462de5c740844a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R3075e9f4c7044606"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="R33c7c19ab0174359"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6dd26396ebd749dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R5d5cd89e9d504e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="Rb47230b1128648ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R295c429d340f4970"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="Rdf3a1f44a89c4eb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R4ab9b6ab14c04162"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Ra4588d684aff475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="R6665803ec5ed4c80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R0c3d49edbb844ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R5b4180914f734889"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R69e3b3521c5945d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R7142cc815949456c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="R6935e7b333fb4626"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="R571d2fe0358b42be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R6cfe19b9e602463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="Rfdfdead4fd6a4e62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,7 +370,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R375385ade1fc40dc"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra7248c847ec549c7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1033,7 +1033,7 @@
     <x:mergeCell ref="A4:H4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15bc2bb6e9a84f6b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R576e7f938927465d"/>
 </x:worksheet>
 </file>
 
@@ -29087,13 +29087,11 @@
         </x:is>
       </x:c>
       <x:c r="D16" s="40" t="n"/>
-      <x:c r="E16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EXPANDING</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F16" s="40" t="b">
-        <x:v>0</x:v>
+      <x:c r="E16" s="40" t="str">
+        <x:v>NON_EXPANDING</x:v>
+      </x:c>
+      <x:c r="F16" s="40" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G16" s="40" t="inlineStr">
         <x:is>
@@ -29131,13 +29129,11 @@
         </x:is>
       </x:c>
       <x:c r="D17" s="40" t="n"/>
-      <x:c r="E17" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EXPANDING</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F17" s="40" t="b">
-        <x:v>0</x:v>
+      <x:c r="E17" s="40" t="str">
+        <x:v>NON_EXPANDING</x:v>
+      </x:c>
+      <x:c r="F17" s="40" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G17" s="40" t="inlineStr">
         <x:is>
@@ -29175,13 +29171,11 @@
         </x:is>
       </x:c>
       <x:c r="D18" s="40" t="n"/>
-      <x:c r="E18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EXPANDING</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F18" s="40" t="b">
-        <x:v>0</x:v>
+      <x:c r="E18" s="40" t="str">
+        <x:v>NON_EXPANDING</x:v>
+      </x:c>
+      <x:c r="F18" s="40" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="40" t="inlineStr">
         <x:is>
@@ -29219,13 +29213,11 @@
         </x:is>
       </x:c>
       <x:c r="D19" s="40" t="n"/>
-      <x:c r="E19" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EXPANDING</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F19" s="40" t="b">
-        <x:v>0</x:v>
+      <x:c r="E19" s="40" t="str">
+        <x:v>NON_EXPANDING</x:v>
+      </x:c>
+      <x:c r="F19" s="40" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G19" s="40" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
codex: wire inclusive Ninth coke and blast targets
Verification: generate/Stages 1-2 completed; data_convert/Stage 3 processed 21 Ninth economies with 100% mapped-source preservation and max drift 1.164e-10; 76 focused tests passed. Detailed standalone rows remain by the current generic NON_EXPANDING contract and are recorded as a human policy decision.
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6dd26396ebd749dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R5d5cd89e9d504e69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="Rb47230b1128648ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R295c429d340f4970"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="Rdf3a1f44a89c4eb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R4ab9b6ab14c04162"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Ra4588d684aff475b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="R6665803ec5ed4c80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R0c3d49edbb844ee7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R5b4180914f734889"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R69e3b3521c5945d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R7142cc815949456c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="R6935e7b333fb4626"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="R571d2fe0358b42be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R6cfe19b9e602463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="Rfdfdead4fd6a4e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0d44505151894ae6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R4b4637099320463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R6ddd7c6106d54d2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R4b6359d0cc324860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="Rd4e028887ee14667"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Rfa7c33ac459946b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rb35f166400a042a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Re0d16b89ea7545f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="Rd0f07503cf6e4265"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="Reda3d4e732504da1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="Ra25dca551fa94509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R8885bad933724c3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="Rab7d80b4ea824991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Rff9246e9deb540d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="Re605ae540edd450e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="Rab0ab9a62fb644aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,7 +370,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra7248c847ec549c7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R72544f2dae924895"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1033,7 +1033,7 @@
     <x:mergeCell ref="A4:H4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R576e7f938927465d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f7bb38f44754f84"/>
 </x:worksheet>
 </file>
 
@@ -37789,1567 +37789,1037 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="42" customFormat="1" ht="34" customHeight="1">
-      <x:c r="A1" s="25" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ninth_sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="25" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">esto_flow</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" s="25" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">esto_dataset_scope</x:t>
-        </x:is>
+      <x:c r="A1" s="25" t="str">
+        <x:v>ninth_sector</x:v>
+      </x:c>
+      <x:c r="B1" s="25" t="str">
+        <x:v>esto_flow</x:v>
+      </x:c>
+      <x:c r="C1" s="25" t="str">
+        <x:v>esto_dataset_scope</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="39" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">01_production</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="39" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">01 Production</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" s="39" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A2" s="39" t="str">
+        <x:v>01_production</x:v>
+      </x:c>
+      <x:c r="B2" s="39" t="str">
+        <x:v>01 Production</x:v>
+      </x:c>
+      <x:c r="C2" s="39" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">02_imports</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">02 Imports</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A3" s="40" t="str">
+        <x:v>02_imports</x:v>
+      </x:c>
+      <x:c r="B3" s="40" t="str">
+        <x:v>02 Imports</x:v>
+      </x:c>
+      <x:c r="C3" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">03_exports</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">03 Exports</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A4" s="40" t="str">
+        <x:v>03_exports</x:v>
+      </x:c>
+      <x:c r="B4" s="40" t="str">
+        <x:v>03 Exports</x:v>
+      </x:c>
+      <x:c r="C4" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">04-05 International transport (bunkers)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">04-05 International transport (bunkers)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A5" s="40" t="str">
+        <x:v>04-05 International transport (bunkers)</x:v>
+      </x:c>
+      <x:c r="B5" s="40" t="str">
+        <x:v>04-05 International transport (bunkers)</x:v>
+      </x:c>
+      <x:c r="C5" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">04_international_marine_bunkers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">04 International marine bunkers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A6" s="40" t="str">
+        <x:v>04_international_marine_bunkers</x:v>
+      </x:c>
+      <x:c r="B6" s="40" t="str">
+        <x:v>04 International marine bunkers</x:v>
+      </x:c>
+      <x:c r="C6" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">05_international_aviation_bunkers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">05 International aviation bunkers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C7" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A7" s="40" t="str">
+        <x:v>05_international_aviation_bunkers</x:v>
+      </x:c>
+      <x:c r="B7" s="40" t="str">
+        <x:v>05 International aviation bunkers</x:v>
+      </x:c>
+      <x:c r="C7" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">07_total_primary_energy_supply</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">07 Total primary energy supply</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C8" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A8" s="40" t="str">
+        <x:v>07_total_primary_energy_supply</x:v>
+      </x:c>
+      <x:c r="B8" s="40" t="str">
+        <x:v>07 Total primary energy supply</x:v>
+      </x:c>
+      <x:c r="C8" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08_transfers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">08 Transfers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C9" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A9" s="40" t="str">
+        <x:v>08_transfers</x:v>
+      </x:c>
+      <x:c r="B9" s="40" t="str">
+        <x:v>08 Transfers</x:v>
+      </x:c>
+      <x:c r="C9" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_01-09_02,09_x Power sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.01-09.02 Power sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C10" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A10" s="40" t="str">
+        <x:v>09_01-09_02,09_x Power sector</x:v>
+      </x:c>
+      <x:c r="B10" s="40" t="str">
+        <x:v>09.01-09.02 Power sector</x:v>
+      </x:c>
+      <x:c r="C10" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_01_electricity_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.01.01,09.02.01 Electricity plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C11" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A11" s="40" t="str">
+        <x:v>09_01_electricity_plants</x:v>
+      </x:c>
+      <x:c r="B11" s="40" t="str">
+        <x:v>09.01.01,09.02.01 Electricity plants</x:v>
+      </x:c>
+      <x:c r="C11" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_02_chp_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.01.02,09.02.02 CHP plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A12" s="40" t="str">
+        <x:v>09_02_chp_plants</x:v>
+      </x:c>
+      <x:c r="B12" s="40" t="str">
+        <x:v>09.01.02,09.02.02 CHP plants</x:v>
+      </x:c>
+      <x:c r="C12" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_02_chp_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.01.02.01 Coal CHP</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C13" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ESTO_EXTENDED</x:t>
-        </x:is>
+      <x:c r="A13" s="40" t="str">
+        <x:v>09_02_chp_plants</x:v>
+      </x:c>
+      <x:c r="B13" s="40" t="str">
+        <x:v>09.01.02.01 Coal CHP</x:v>
+      </x:c>
+      <x:c r="C13" s="40" t="str">
+        <x:v>ESTO_EXTENDED</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_04_electric_boilers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B14" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.04 Electric boilers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C14" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A14" s="40" t="str">
+        <x:v>09_04_electric_boilers</x:v>
+      </x:c>
+      <x:c r="B14" s="40" t="str">
+        <x:v>09.04 Electric boilers</x:v>
+      </x:c>
+      <x:c r="C14" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_05_chemical_heat_for_electricity_production</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.05 Chemical heat for electricity production</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C15" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A15" s="40" t="str">
+        <x:v>09_05_chemical_heat_for_electricity_production</x:v>
+      </x:c>
+      <x:c r="B15" s="40" t="str">
+        <x:v>09.05 Chemical heat for electricity production</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_06_01_gas_works_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.06.01 Gas works plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C16" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A16" s="40" t="str">
+        <x:v>09_06_01_gas_works_plants</x:v>
+      </x:c>
+      <x:c r="B16" s="40" t="str">
+        <x:v>09.06.01 Gas works plants</x:v>
+      </x:c>
+      <x:c r="C16" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_06_01_gas_works_plants_incl_own_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.06.01 Gas works plants (including own use)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C17" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A17" s="40" t="str">
+        <x:v>09_06_01_gas_works_plants_incl_own_use</x:v>
+      </x:c>
+      <x:c r="B17" s="40" t="str">
+        <x:v>09.06.01 Gas works plants (including own use)</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_06_02_liquefaction_regasification_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.06.02 Liquefaction/regasification plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C18" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A18" s="40" t="str">
+        <x:v>09_06_02_liquefaction_regasification_plants</x:v>
+      </x:c>
+      <x:c r="B18" s="40" t="str">
+        <x:v>09.06.02 Liquefaction/regasification plants</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_06_02_liquefaction_regasification_plants_incl_own_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B19" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.06.02 Liquefaction/regasification plants (including own use)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C19" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A19" s="40" t="str">
+        <x:v>09_06_02_liquefaction_regasification_plants_incl_own_use</x:v>
+      </x:c>
+      <x:c r="B19" s="40" t="str">
+        <x:v>09.06.02 Liquefaction/regasification plants (including own use)</x:v>
+      </x:c>
+      <x:c r="C19" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_06_gas_processing_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B20" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.06 Gas processing plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C20" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A20" s="40" t="str">
+        <x:v>09_06_gas_processing_plants</x:v>
+      </x:c>
+      <x:c r="B20" s="40" t="str">
+        <x:v>09.06 Gas processing plants</x:v>
+      </x:c>
+      <x:c r="C20" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_06_gas_processing_plants_incl_own_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B21" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.06 Gas processing plants (including own use)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C21" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A21" s="40" t="str">
+        <x:v>09_06_gas_processing_plants_incl_own_use</x:v>
+      </x:c>
+      <x:c r="B21" s="40" t="str">
+        <x:v>09.06 Gas processing plants (including own use)</x:v>
+      </x:c>
+      <x:c r="C21" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_07_oil_refineries</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B22" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.07 Oil refineries</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C22" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A22" s="40" t="str">
+        <x:v>09_07_oil_refineries</x:v>
+      </x:c>
+      <x:c r="B22" s="40" t="str">
+        <x:v>09.07 Oil refineries</x:v>
+      </x:c>
+      <x:c r="C22" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_07_oil_refineries_incl_own_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B23" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.07 Oil refineries (including own use)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C23" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A23" s="40" t="str">
+        <x:v>09_07_oil_refineries_incl_own_use</x:v>
+      </x:c>
+      <x:c r="B23" s="40" t="str">
+        <x:v>09.07 Oil refineries (including own use)</x:v>
+      </x:c>
+      <x:c r="C23" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_08_coal_transformation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B24" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.08 Coal transformation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C24" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A24" s="40" t="str">
+        <x:v>09_08_coal_transformation</x:v>
+      </x:c>
+      <x:c r="B24" s="40" t="str">
+        <x:v>09.08 Coal transformation</x:v>
+      </x:c>
+      <x:c r="C24" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_08_coal_transformation_incl_own_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B25" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.08 Coal transformation (including own use)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C25" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A25" s="40" t="str">
+        <x:v>09_08_coal_transformation_incl_own_use</x:v>
+      </x:c>
+      <x:c r="B25" s="40" t="str">
+        <x:v>09.08 Coal transformation (including own use)</x:v>
+      </x:c>
+      <x:c r="C25" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_09_petrochemical_industry</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.09 Petrochemical industry</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A26" s="40" t="str">
+        <x:v>09_08_01_coke_ovens_incl_own_use</x:v>
+      </x:c>
+      <x:c r="B26" s="40" t="str">
+        <x:v>09.08.01 Coke ovens (including own use)</x:v>
+      </x:c>
+      <x:c r="C26" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_11_charcoal_processing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.11 Charcoal processing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A27" s="40" t="str">
+        <x:v>09_08_02_blast_furnaces_incl_own_use</x:v>
+      </x:c>
+      <x:c r="B27" s="40" t="str">
+        <x:v>09.08.02 Blast furnaces (including own use)</x:v>
+      </x:c>
+      <x:c r="C27" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_12_nonspecified_transformation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.12 Non-specified transformation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A28" s="40" t="str">
+        <x:v>09_09_petrochemical_industry</x:v>
+      </x:c>
+      <x:c r="B28" s="40" t="str">
+        <x:v>09.09 Petrochemical industry</x:v>
+      </x:c>
+      <x:c r="C28" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_13_01_electrolysers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B29" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.13.01 Electrolysers</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C29" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A29" s="40" t="str">
+        <x:v>09_11_charcoal_processing</x:v>
+      </x:c>
+      <x:c r="B29" s="40" t="str">
+        <x:v>09.11 Charcoal processing</x:v>
+      </x:c>
+      <x:c r="C29" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_13_02_smr_wo_ccs</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B30" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.13.02 SMR wo CCS</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C30" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A30" s="40" t="str">
+        <x:v>09_12_nonspecified_transformation</x:v>
+      </x:c>
+      <x:c r="B30" s="40" t="str">
+        <x:v>09.12 Non-specified transformation</x:v>
+      </x:c>
+      <x:c r="C30" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_13_03_smr_w_ccs</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.13.03 SMR w CCS</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C31" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A31" s="40" t="str">
+        <x:v>09_13_01_electrolysers</x:v>
+      </x:c>
+      <x:c r="B31" s="40" t="str">
+        <x:v>09.13.01 Electrolysers</x:v>
+      </x:c>
+      <x:c r="C31" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_13_hydrogen_transformation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.13 Hydrogen transformation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A32" s="40" t="str">
+        <x:v>09_13_02_smr_wo_ccs</x:v>
+      </x:c>
+      <x:c r="B32" s="40" t="str">
+        <x:v>09.13.02 SMR wo CCS</x:v>
+      </x:c>
+      <x:c r="C32" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_total_transformation_sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09 Total transformation sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A33" s="40" t="str">
+        <x:v>09_13_03_smr_w_ccs</x:v>
+      </x:c>
+      <x:c r="B33" s="40" t="str">
+        <x:v>09.13.03 SMR w CCS</x:v>
+      </x:c>
+      <x:c r="C33" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_12_nonspecified_transformation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.03 Heat pumps</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A34" s="40" t="str">
+        <x:v>09_13_hydrogen_transformation</x:v>
+      </x:c>
+      <x:c r="B34" s="40" t="str">
+        <x:v>09.13 Hydrogen transformation</x:v>
+      </x:c>
+      <x:c r="C34" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09_x_heat_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.01.03,09.02.03 Heat plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A35" s="40" t="str">
+        <x:v>09_total_transformation_sector</x:v>
+      </x:c>
+      <x:c r="B35" s="40" t="str">
+        <x:v>09 Total transformation sector</x:v>
+      </x:c>
+      <x:c r="C35" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_01_electricity_chp_and_heat_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B36" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.01 Electricity, CHP and heat plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C36" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A36" s="40" t="str">
+        <x:v>09_12_nonspecified_transformation</x:v>
+      </x:c>
+      <x:c r="B36" s="40" t="str">
+        <x:v>09.03 Heat pumps</x:v>
+      </x:c>
+      <x:c r="C36" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_02_gas_works_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B37" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.02 Gas works plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C37" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A37" s="40" t="str">
+        <x:v>09_x_heat_plants</x:v>
+      </x:c>
+      <x:c r="B37" s="40" t="str">
+        <x:v>09.01.03,09.02.03 Heat plants</x:v>
+      </x:c>
+      <x:c r="C37" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_03_liquefaction_regasification_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B38" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.03 Liquefaction/regasification plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C38" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A38" s="40" t="str">
+        <x:v>10_01_01_electricity_chp_and_heat_plants</x:v>
+      </x:c>
+      <x:c r="B38" s="40" t="str">
+        <x:v>10.01.01 Electricity, CHP and heat plants</x:v>
+      </x:c>
+      <x:c r="C38" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_05_coke_ovens</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B39" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.05 Coke ovens</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C39" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A39" s="40" t="str">
+        <x:v>10_01_02_gas_works_plants</x:v>
+      </x:c>
+      <x:c r="B39" s="40" t="str">
+        <x:v>10.01.02 Gas works plants</x:v>
+      </x:c>
+      <x:c r="C39" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_06_coal_mines</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B40" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.06 Coal mines</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C40" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A40" s="40" t="str">
+        <x:v>10_01_03_liquefaction_regasification_plants</x:v>
+      </x:c>
+      <x:c r="B40" s="40" t="str">
+        <x:v>10.01.03 Liquefaction/regasification plants</x:v>
+      </x:c>
+      <x:c r="C40" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_07_blast_furnaces</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B41" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.07 Blast furnaces</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C41" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A41" s="40" t="str">
+        <x:v>10_01_05_coke_ovens</x:v>
+      </x:c>
+      <x:c r="B41" s="40" t="str">
+        <x:v>10.01.05 Coke ovens</x:v>
+      </x:c>
+      <x:c r="C41" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_11_oil_refineries</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B42" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.11 Oil refineries</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C42" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A42" s="40" t="str">
+        <x:v>10_01_06_coal_mines</x:v>
+      </x:c>
+      <x:c r="B42" s="40" t="str">
+        <x:v>10.01.06 Coal mines</x:v>
+      </x:c>
+      <x:c r="C42" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_12_oil_and_gas_extraction</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B43" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.12 Oil and gas extraction</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C43" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A43" s="40" t="str">
+        <x:v>10_01_07_blast_furnaces</x:v>
+      </x:c>
+      <x:c r="B43" s="40" t="str">
+        <x:v>10.01.07 Blast furnaces</x:v>
+      </x:c>
+      <x:c r="C43" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_13_pump_storage_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B44" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.13 Pump storage plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C44" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A44" s="40" t="str">
+        <x:v>10_01_11_oil_refineries</x:v>
+      </x:c>
+      <x:c r="B44" s="40" t="str">
+        <x:v>10.01.11 Oil refineries</x:v>
+      </x:c>
+      <x:c r="C44" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_17_nonspecified_own_uses</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B45" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.17 Non-specified own uses</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C45" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A45" s="40" t="str">
+        <x:v>10_01_12_oil_and_gas_extraction</x:v>
+      </x:c>
+      <x:c r="B45" s="40" t="str">
+        <x:v>10.01.12 Oil and gas extraction</x:v>
+      </x:c>
+      <x:c r="C45" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_01_19_hydrogen_transformation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B46" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.01.19 Hydrogen transformation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C46" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A46" s="40" t="str">
+        <x:v>10_01_13_pump_storage_plants</x:v>
+      </x:c>
+      <x:c r="B46" s="40" t="str">
+        <x:v>10.01.13 Pump storage plants</x:v>
+      </x:c>
+      <x:c r="C46" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10_02_transmission_and_distribution_losses</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B47" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10.02 Transmission and distribution losses</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C47" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A47" s="40" t="str">
+        <x:v>10_01_17_nonspecified_own_uses</x:v>
+      </x:c>
+      <x:c r="B47" s="40" t="str">
+        <x:v>10.01.17 Non-specified own uses</x:v>
+      </x:c>
+      <x:c r="C47" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">12_total_final_consumption</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B48" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">12 Total final consumption</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C48" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A48" s="40" t="str">
+        <x:v>10_01_19_hydrogen_transformation</x:v>
+      </x:c>
+      <x:c r="B48" s="40" t="str">
+        <x:v>10.01.19 Hydrogen transformation</x:v>
+      </x:c>
+      <x:c r="C48" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">13_total_final_energy_consumption</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B49" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">13 Total final energy consumption</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C49" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A49" s="40" t="str">
+        <x:v>10_02_transmission_and_distribution_losses</x:v>
+      </x:c>
+      <x:c r="B49" s="40" t="str">
+        <x:v>10.02 Transmission and distribution losses</x:v>
+      </x:c>
+      <x:c r="C49" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_01_mining_and_quarrying</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B50" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.01 Mining and quarrying</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C50" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A50" s="40" t="str">
+        <x:v>12_total_final_consumption</x:v>
+      </x:c>
+      <x:c r="B50" s="40" t="str">
+        <x:v>12 Total final consumption</x:v>
+      </x:c>
+      <x:c r="C50" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_02_construction</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B51" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.02 Construction</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C51" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A51" s="40" t="str">
+        <x:v>13_total_final_energy_consumption</x:v>
+      </x:c>
+      <x:c r="B51" s="40" t="str">
+        <x:v>13 Total final energy consumption</x:v>
+      </x:c>
+      <x:c r="C51" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_01_iron_and_steel</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B52" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.01 Iron and steel</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C52" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A52" s="40" t="str">
+        <x:v>14_01_mining_and_quarrying</x:v>
+      </x:c>
+      <x:c r="B52" s="40" t="str">
+        <x:v>14.01 Mining and quarrying</x:v>
+      </x:c>
+      <x:c r="C52" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_02_chemical_incl_petrochemical</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B53" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.02 Chemical (incl. petrochemical)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C53" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A53" s="40" t="str">
+        <x:v>14_02_construction</x:v>
+      </x:c>
+      <x:c r="B53" s="40" t="str">
+        <x:v>14.02 Construction</x:v>
+      </x:c>
+      <x:c r="C53" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_03_non_ferrous_metals</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B54" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.03 Non ferrous metals</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C54" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A54" s="40" t="str">
+        <x:v>14_03_01_iron_and_steel</x:v>
+      </x:c>
+      <x:c r="B54" s="40" t="str">
+        <x:v>14.03.01 Iron and steel</x:v>
+      </x:c>
+      <x:c r="C54" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_04_nonmetallic_mineral_products</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B55" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.04 Non-metallic mineral products</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C55" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A55" s="40" t="str">
+        <x:v>14_03_02_chemical_incl_petrochemical</x:v>
+      </x:c>
+      <x:c r="B55" s="40" t="str">
+        <x:v>14.03.02 Chemical (incl. petrochemical)</x:v>
+      </x:c>
+      <x:c r="C55" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_05_transportation_equipment</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B56" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.05 Transportation equipment</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C56" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A56" s="40" t="str">
+        <x:v>14_03_03_non_ferrous_metals</x:v>
+      </x:c>
+      <x:c r="B56" s="40" t="str">
+        <x:v>14.03.03 Non ferrous metals</x:v>
+      </x:c>
+      <x:c r="C56" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_06_machinery</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B57" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.06 Machinery</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C57" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A57" s="40" t="str">
+        <x:v>14_03_04_nonmetallic_mineral_products</x:v>
+      </x:c>
+      <x:c r="B57" s="40" t="str">
+        <x:v>14.03.04 Non-metallic mineral products</x:v>
+      </x:c>
+      <x:c r="C57" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_07_food_beverages_and_tobacco</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B58" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.07 Food, beverages and tobacco</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C58" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A58" s="40" t="str">
+        <x:v>14_03_05_transportation_equipment</x:v>
+      </x:c>
+      <x:c r="B58" s="40" t="str">
+        <x:v>14.03.05 Transportation equipment</x:v>
+      </x:c>
+      <x:c r="C58" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_08_pulp_paper_and_printing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B59" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.08 Pulp, paper and printing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C59" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A59" s="40" t="str">
+        <x:v>14_03_06_machinery</x:v>
+      </x:c>
+      <x:c r="B59" s="40" t="str">
+        <x:v>14.03.06 Machinery</x:v>
+      </x:c>
+      <x:c r="C59" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_09_wood_and_wood_products</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B60" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.09 Wood and wood products</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C60" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A60" s="40" t="str">
+        <x:v>14_03_07_food_beverages_and_tobacco</x:v>
+      </x:c>
+      <x:c r="B60" s="40" t="str">
+        <x:v>14.03.07 Food, beverages and tobacco</x:v>
+      </x:c>
+      <x:c r="C60" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
-      <x:c r="A61" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_10_textiles_and_leather</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B61" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.10 Textiles and leather</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C61" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A61" s="40" t="str">
+        <x:v>14_03_08_pulp_paper_and_printing</x:v>
+      </x:c>
+      <x:c r="B61" s="40" t="str">
+        <x:v>14.03.08 Pulp, paper and printing</x:v>
+      </x:c>
+      <x:c r="C61" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_11_nonspecified_industry</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B62" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03.11 Non-specified industry</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C62" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A62" s="40" t="str">
+        <x:v>14_03_09_wood_and_wood_products</x:v>
+      </x:c>
+      <x:c r="B62" s="40" t="str">
+        <x:v>14.03.09 Wood and wood products</x:v>
+      </x:c>
+      <x:c r="C62" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_03_manufacturing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B63" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14.03 Manufacturing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C63" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A63" s="40" t="str">
+        <x:v>14_03_10_textiles_and_leather</x:v>
+      </x:c>
+      <x:c r="B63" s="40" t="str">
+        <x:v>14.03.10 Textiles and leather</x:v>
+      </x:c>
+      <x:c r="C63" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14_industry_sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B64" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14 Industry sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C64" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A64" s="40" t="str">
+        <x:v>14_03_11_nonspecified_industry</x:v>
+      </x:c>
+      <x:c r="B64" s="40" t="str">
+        <x:v>14.03.11 Non-specified industry</x:v>
+      </x:c>
+      <x:c r="C64" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15_01,15_03-15_06 Transport non-road</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B65" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15.01,15.03-15.06 Transport non-road</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C65" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A65" s="40" t="str">
+        <x:v>14_03_manufacturing</x:v>
+      </x:c>
+      <x:c r="B65" s="40" t="str">
+        <x:v>14.03 Manufacturing</x:v>
+      </x:c>
+      <x:c r="C65" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15_01_domestic_air_transport</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B66" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15.01 Domestic air transport</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C66" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A66" s="40" t="str">
+        <x:v>14_industry_sector</x:v>
+      </x:c>
+      <x:c r="B66" s="40" t="str">
+        <x:v>14 Industry sector</x:v>
+      </x:c>
+      <x:c r="C66" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15_02_road</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B67" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15.02 Road</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C67" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A67" s="40" t="str">
+        <x:v>15_01,15_03-15_06 Transport non-road</x:v>
+      </x:c>
+      <x:c r="B67" s="40" t="str">
+        <x:v>15.01,15.03-15.06 Transport non-road</x:v>
+      </x:c>
+      <x:c r="C67" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
-      <x:c r="A68" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15_03_rail</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B68" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15.03 Rail</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C68" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A68" s="40" t="str">
+        <x:v>15_01_domestic_air_transport</x:v>
+      </x:c>
+      <x:c r="B68" s="40" t="str">
+        <x:v>15.01 Domestic air transport</x:v>
+      </x:c>
+      <x:c r="C68" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
-      <x:c r="A69" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15_04_domestic_navigation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B69" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15.04 Domestic navigation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C69" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A69" s="40" t="str">
+        <x:v>15_02_road</x:v>
+      </x:c>
+      <x:c r="B69" s="40" t="str">
+        <x:v>15.02 Road</x:v>
+      </x:c>
+      <x:c r="C69" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
-      <x:c r="A70" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15_05_pipeline_transport</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B70" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15.05 Pipeline transport</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C70" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A70" s="40" t="str">
+        <x:v>15_03_rail</x:v>
+      </x:c>
+      <x:c r="B70" s="40" t="str">
+        <x:v>15.03 Rail</x:v>
+      </x:c>
+      <x:c r="C70" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
-      <x:c r="A71" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15_06_nonspecified_transport</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B71" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15.06 Non-specified transport</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C71" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A71" s="40" t="str">
+        <x:v>15_04_domestic_navigation</x:v>
+      </x:c>
+      <x:c r="B71" s="40" t="str">
+        <x:v>15.04 Domestic navigation</x:v>
+      </x:c>
+      <x:c r="C71" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
-      <x:c r="A72" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15_transport_sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B72" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15 Transport sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C72" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A72" s="40" t="str">
+        <x:v>15_05_pipeline_transport</x:v>
+      </x:c>
+      <x:c r="B72" s="40" t="str">
+        <x:v>15.05 Pipeline transport</x:v>
+      </x:c>
+      <x:c r="C72" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
-      <x:c r="A73" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_01_01_commercial_and_public_services</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B73" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.01.99 Commercial and public services unallocated</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C73" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A73" s="40" t="str">
+        <x:v>15_06_nonspecified_transport</x:v>
+      </x:c>
+      <x:c r="B73" s="40" t="str">
+        <x:v>15.06 Non-specified transport</x:v>
+      </x:c>
+      <x:c r="C73" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
-      <x:c r="A74" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_01_01_commercial_and_public_services_incl_datacentres</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B74" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.01 Commercial and public services</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C74" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A74" s="40" t="str">
+        <x:v>15_transport_sector</x:v>
+      </x:c>
+      <x:c r="B74" s="40" t="str">
+        <x:v>15 Transport sector</x:v>
+      </x:c>
+      <x:c r="C74" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
-      <x:c r="A75" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_01_02_residential</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B75" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.02 Residential</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C75" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A75" s="40" t="str">
+        <x:v>16_01_01_commercial_and_public_services</x:v>
+      </x:c>
+      <x:c r="B75" s="40" t="str">
+        <x:v>16.01.99 Commercial and public services unallocated</x:v>
+      </x:c>
+      <x:c r="C75" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
-      <x:c r="A76" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_01_03_ai_training</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B76" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.01.01 Datacentres</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C76" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A76" s="40" t="str">
+        <x:v>16_01_01_commercial_and_public_services_incl_datacentres</x:v>
+      </x:c>
+      <x:c r="B76" s="40" t="str">
+        <x:v>16.01 Commercial and public services</x:v>
+      </x:c>
+      <x:c r="C76" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
-      <x:c r="A77" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_01_04_traditional_data_centres</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B77" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.01.01 Datacentres</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C77" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A77" s="40" t="str">
+        <x:v>16_01_02_residential</x:v>
+      </x:c>
+      <x:c r="B77" s="40" t="str">
+        <x:v>16.02 Residential</x:v>
+      </x:c>
+      <x:c r="C77" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B78" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C78" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A78" s="40" t="str">
+        <x:v>16_01_03_ai_training</x:v>
+      </x:c>
+      <x:c r="B78" s="40" t="str">
+        <x:v>16.01.01 Datacentres</x:v>
+      </x:c>
+      <x:c r="C78" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02_agriculture_and_fishing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B79" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.04 Agriculture and fishing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C79" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A79" s="40" t="str">
+        <x:v>16_01_04_traditional_data_centres</x:v>
+      </x:c>
+      <x:c r="B79" s="40" t="str">
+        <x:v>16.01.01 Datacentres</x:v>
+      </x:c>
+      <x:c r="C79" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_05_nonspecified_others</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B80" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.05 Non-specified others</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C80" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A80" s="40" t="str">
+        <x:v>16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="B80" s="40" t="str">
+        <x:v>16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="C80" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_other_sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B81" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16 Other sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C81" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A81" s="40" t="str">
+        <x:v>16_02_agriculture_and_fishing</x:v>
+      </x:c>
+      <x:c r="B81" s="40" t="str">
+        <x:v>16.03-16.04 Agriculture and fishing</x:v>
+      </x:c>
+      <x:c r="C81" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17_nonenergy_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B82" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17 Non-energy use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C82" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A82" s="40" t="str">
+        <x:v>16_05_nonspecified_others</x:v>
+      </x:c>
+      <x:c r="B82" s="40" t="str">
+        <x:v>16.05 Non-specified others</x:v>
+      </x:c>
+      <x:c r="C82" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
-      <x:c r="A83" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18_01_electricity_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B83" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18.01 MAP electricity plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C83" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A83" s="40" t="str">
+        <x:v>16_other_sector</x:v>
+      </x:c>
+      <x:c r="B83" s="40" t="str">
+        <x:v>16 Other sector</x:v>
+      </x:c>
+      <x:c r="C83" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
-      <x:c r="A84" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18_01_electricity_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B84" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18.02 MAP CHP plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C84" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A84" s="40" t="str">
+        <x:v>17_nonenergy_use</x:v>
+      </x:c>
+      <x:c r="B84" s="40" t="str">
+        <x:v>17 Non-energy use</x:v>
+      </x:c>
+      <x:c r="C84" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
-      <x:c r="A85" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18_01_electricity_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B85" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18.03 AP electricity plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C85" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A85" s="40" t="str">
+        <x:v>18_01_electricity_plants</x:v>
+      </x:c>
+      <x:c r="B85" s="40" t="str">
+        <x:v>18.01 MAP electricity plants</x:v>
+      </x:c>
+      <x:c r="C85" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
-      <x:c r="A86" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18_02_chp_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B86" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18.04 AP CHP plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C86" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A86" s="40" t="str">
+        <x:v>18_01_electricity_plants</x:v>
+      </x:c>
+      <x:c r="B86" s="40" t="str">
+        <x:v>18.02 MAP CHP plants</x:v>
+      </x:c>
+      <x:c r="C86" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
-      <x:c r="A87" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18_electricity_output_in_gwh</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B87" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">18 Electricity output in GWh</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C87" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A87" s="40" t="str">
+        <x:v>18_01_electricity_plants</x:v>
+      </x:c>
+      <x:c r="B87" s="40" t="str">
+        <x:v>18.03 AP electricity plants</x:v>
+      </x:c>
+      <x:c r="C87" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
-      <x:c r="A88" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19_01_chp_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B88" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19.01 MAP CHP plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C88" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A88" s="40" t="str">
+        <x:v>18_02_chp_plants</x:v>
+      </x:c>
+      <x:c r="B88" s="40" t="str">
+        <x:v>18.04 AP CHP plants</x:v>
+      </x:c>
+      <x:c r="C88" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
-      <x:c r="A89" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19_01_chp_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B89" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19.03 AP CHP plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C89" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A89" s="40" t="str">
+        <x:v>18_electricity_output_in_gwh</x:v>
+      </x:c>
+      <x:c r="B89" s="40" t="str">
+        <x:v>18 Electricity output in GWh</x:v>
+      </x:c>
+      <x:c r="C89" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
-      <x:c r="A90" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19_02_heat_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B90" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19.02 MAP heat plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C90" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A90" s="40" t="str">
+        <x:v>19_01_chp_plants</x:v>
+      </x:c>
+      <x:c r="B90" s="40" t="str">
+        <x:v>19.01 MAP CHP plants</x:v>
+      </x:c>
+      <x:c r="C90" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
-      <x:c r="A91" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19_02_heat_plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B91" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19.04 AP heat plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C91" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A91" s="40" t="str">
+        <x:v>19_01_chp_plants</x:v>
+      </x:c>
+      <x:c r="B91" s="40" t="str">
+        <x:v>19.03 AP CHP plants</x:v>
+      </x:c>
+      <x:c r="C91" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
-      <x:c r="A92" s="41" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19_heat_output_in_pj</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B92" s="41" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">19 Heat output in PJ</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C92" s="41" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A92" s="41" t="str">
+        <x:v>19_02_heat_plants</x:v>
+      </x:c>
+      <x:c r="B92" s="41" t="str">
+        <x:v>19.02 MAP heat plants</x:v>
+      </x:c>
+      <x:c r="C92" s="41" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>19_02_heat_plants</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>19.04 AP heat plants</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>BOTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>19_heat_output_in_pj</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>19 Heat output in PJ</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
codex: cut over non-energy demand mapping
Map the clean-slate LEAP Non Energy Use branch directly to flow 17, keep Other sector at 16.03-16.05, add the branch to TFC, disable the former combined subtotal, and regenerate mapping authorities.\n\nValidation: 6 focused tests passed; common ESTO mapped-row total differences max 1.16e-10. Full recursive tree validation was interrupted after core outputs completed because it exceeded available memory.
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0d44505151894ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R4b4637099320463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R6ddd7c6106d54d2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R4b6359d0cc324860"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="Rd4e028887ee14667"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Rfa7c33ac459946b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rb35f166400a042a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Re0d16b89ea7545f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="Rd0f07503cf6e4265"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="Reda3d4e732504da1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="Ra25dca551fa94509"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R8885bad933724c3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="Rab7d80b4ea824991"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Rff9246e9deb540d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="Re605ae540edd450e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="Rab0ab9a62fb644aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rdd80abd5a6224d28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R97489b0115d044ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R83b35ae960534904"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R1ed27f1c81d64ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R68eaf2c58694499b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R7a0f2b592a1c4bdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="R900655755405433e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="Rdafe65d8c169415a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R0d167d64e5a54137"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R946b8fe338594398"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="Rdd0527a5a86f426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="R479d1507fc3a409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="R47c213e8a1da4296"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Rfbd5f9def7d34adc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="Rcb7d355f4e8a4e46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="Re964af885f22468c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,7 +370,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R72544f2dae924895"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0fceabdc21d448ab"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1033,7 +1033,7 @@
     <x:mergeCell ref="A4:H4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f7bb38f44754f84"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4fed3fecfb54ecb"/>
 </x:worksheet>
 </file>
 
@@ -20864,11 +20864,11 @@
       <x:c r="A27" s="40" t="str">
         <x:v>All demand aggregated/Buildings</x:v>
       </x:c>
-      <x:c r="B27" s="40" t="str"/>
+      <x:c r="B27" s="40"/>
       <x:c r="C27" s="40" t="str">
         <x:v>Total final consumption</x:v>
       </x:c>
-      <x:c r="D27" s="40" t="str"/>
+      <x:c r="D27" s="40"/>
       <x:c r="E27" s="40" t="str">
         <x:v>NON_EXPANDING</x:v>
       </x:c>
@@ -20876,14 +20876,14 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G27" s="40" t="str">
-        <x:v>Domestic final-consumption boundary derived from the five All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
+        <x:v>Domestic final-consumption boundary derived from the six All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
       </x:c>
       <x:c r="H27" s="44" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I27" s="40"/>
       <x:c r="J27" s="40" t="str">
-        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector</x:v>
+        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector; All demand aggregated/Non Energy Use</x:v>
       </x:c>
       <x:c r="K27" s="40"/>
       <x:c r="L27" s="40"/>
@@ -20897,11 +20897,11 @@
       <x:c r="A28" s="40" t="str">
         <x:v>All demand aggregated/Industry</x:v>
       </x:c>
-      <x:c r="B28" s="40" t="str"/>
+      <x:c r="B28" s="40"/>
       <x:c r="C28" s="40" t="str">
         <x:v>Total final consumption</x:v>
       </x:c>
-      <x:c r="D28" s="40" t="str"/>
+      <x:c r="D28" s="40"/>
       <x:c r="E28" s="40" t="str">
         <x:v>NON_EXPANDING</x:v>
       </x:c>
@@ -20909,14 +20909,14 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G28" s="40" t="str">
-        <x:v>Domestic final-consumption boundary derived from the five All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
+        <x:v>Domestic final-consumption boundary derived from the six All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
       </x:c>
       <x:c r="H28" s="44" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I28" s="40"/>
       <x:c r="J28" s="40" t="str">
-        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector</x:v>
+        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector; All demand aggregated/Non Energy Use</x:v>
       </x:c>
       <x:c r="K28" s="40"/>
       <x:c r="L28" s="40"/>
@@ -20930,11 +20930,11 @@
       <x:c r="A29" s="40" t="str">
         <x:v>All demand aggregated/Road</x:v>
       </x:c>
-      <x:c r="B29" s="40" t="str"/>
+      <x:c r="B29" s="40"/>
       <x:c r="C29" s="40" t="str">
         <x:v>Total final consumption</x:v>
       </x:c>
-      <x:c r="D29" s="40" t="str"/>
+      <x:c r="D29" s="40"/>
       <x:c r="E29" s="40" t="str">
         <x:v>NON_EXPANDING</x:v>
       </x:c>
@@ -20942,14 +20942,14 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G29" s="40" t="str">
-        <x:v>Domestic final-consumption boundary derived from the five All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
+        <x:v>Domestic final-consumption boundary derived from the six All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
       </x:c>
       <x:c r="H29" s="44" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I29" s="40"/>
       <x:c r="J29" s="40" t="str">
-        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector</x:v>
+        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector; All demand aggregated/Non Energy Use</x:v>
       </x:c>
       <x:c r="K29" s="40"/>
       <x:c r="L29" s="40"/>
@@ -20963,11 +20963,11 @@
       <x:c r="A30" s="40" t="str">
         <x:v>All demand aggregated/Transport non road</x:v>
       </x:c>
-      <x:c r="B30" s="40" t="str"/>
+      <x:c r="B30" s="40"/>
       <x:c r="C30" s="40" t="str">
         <x:v>Total final consumption</x:v>
       </x:c>
-      <x:c r="D30" s="40" t="str"/>
+      <x:c r="D30" s="40"/>
       <x:c r="E30" s="40" t="str">
         <x:v>NON_EXPANDING</x:v>
       </x:c>
@@ -20975,14 +20975,14 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G30" s="40" t="str">
-        <x:v>Domestic final-consumption boundary derived from the five All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
+        <x:v>Domestic final-consumption boundary derived from the six All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
       </x:c>
       <x:c r="H30" s="44" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I30" s="40"/>
       <x:c r="J30" s="40" t="str">
-        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector</x:v>
+        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector; All demand aggregated/Non Energy Use</x:v>
       </x:c>
       <x:c r="K30" s="40"/>
       <x:c r="L30" s="40"/>
@@ -20996,11 +20996,11 @@
       <x:c r="A31" s="40" t="str">
         <x:v>All demand aggregated/Other sector</x:v>
       </x:c>
-      <x:c r="B31" s="40" t="str"/>
+      <x:c r="B31" s="40"/>
       <x:c r="C31" s="40" t="str">
         <x:v>Total final consumption</x:v>
       </x:c>
-      <x:c r="D31" s="40" t="str"/>
+      <x:c r="D31" s="40"/>
       <x:c r="E31" s="40" t="str">
         <x:v>NON_EXPANDING</x:v>
       </x:c>
@@ -21008,14 +21008,14 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G31" s="40" t="str">
-        <x:v>Domestic final-consumption boundary derived from the five All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
+        <x:v>Domestic final-consumption boundary derived from the six All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
       </x:c>
       <x:c r="H31" s="44" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I31" s="40"/>
       <x:c r="J31" s="40" t="str">
-        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector</x:v>
+        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector; All demand aggregated/Non Energy Use</x:v>
       </x:c>
       <x:c r="K31" s="40"/>
       <x:c r="L31" s="40"/>
@@ -22855,6 +22855,39 @@
       </x:c>
       <x:c r="N84"/>
       <x:c r="O84"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>All demand aggregated/Non Energy Use</x:v>
+      </x:c>
+      <x:c r="B85"/>
+      <x:c r="C85" t="str">
+        <x:v>Total final consumption</x:v>
+      </x:c>
+      <x:c r="D85"/>
+      <x:c r="E85" t="str">
+        <x:v>NON_EXPANDING</x:v>
+      </x:c>
+      <x:c r="F85" s="46" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>Domestic final-consumption boundary derived from the six All demand aggregated child branches. The parent is not used because it also contains International transport (bunkers).</x:v>
+      </x:c>
+      <x:c r="H85" s="46" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I85"/>
+      <x:c r="J85" t="str">
+        <x:v>All demand aggregated/Buildings; All demand aggregated/Industry; All demand aggregated/Road; All demand aggregated/Transport non road; All demand aggregated/Other sector; All demand aggregated/Non Energy Use</x:v>
+      </x:c>
+      <x:c r="K85"/>
+      <x:c r="L85"/>
+      <x:c r="M85"/>
+      <x:c r="N85"/>
+      <x:c r="O85" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -24430,239 +24463,159 @@
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03 Agriculture</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B32" s="40" t="n"/>
-      <x:c r="C32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D32" s="40" t="n"/>
-      <x:c r="E32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DETACHED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F32" s="40" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Detached comparison boundary for LEAP All demand aggregated/Other sector. Sums agriculture, fishing, non-specified others, and non-energy use without making flow 17 a child of flow 16 or changing the detailed LEAP structure.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MIXED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03 Agriculture; 16.04 Fishing; 16.05 Non-specified others; 17 Non-energy use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">other_sector_comparison</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">all_demand_aggregated_esto_rollup_rules</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M32" s="40" t="n"/>
-      <x:c r="N32" s="40" t="n"/>
-      <x:c r="O32" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A32" s="40" t="str">
+        <x:v>16.03 Agriculture</x:v>
+      </x:c>
+      <x:c r="B32" s="40"/>
+      <x:c r="C32" s="40" t="str">
+        <x:v>16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="D32" s="40"/>
+      <x:c r="E32" s="40" t="str">
+        <x:v>DETACHED</x:v>
+      </x:c>
+      <x:c r="F32" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G32" s="40" t="str">
+        <x:v>Disabled after the global clean-slate cutover: Non-energy use is mapped as its own flow 17 branch, so the former combined Other-sector subtotal must not be generated.</x:v>
+      </x:c>
+      <x:c r="H32" s="40" t="str">
+        <x:v>MIXED</x:v>
+      </x:c>
+      <x:c r="I32" s="40" t="str">
+        <x:v>16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="J32" s="40" t="str">
+        <x:v>16.03 Agriculture; 16.04 Fishing; 16.05 Non-specified others; 17 Non-energy use</x:v>
+      </x:c>
+      <x:c r="K32" s="40" t="str">
+        <x:v>other_sector_comparison</x:v>
+      </x:c>
+      <x:c r="L32" s="40" t="str">
+        <x:v>all_demand_aggregated_esto_rollup_rules</x:v>
+      </x:c>
+      <x:c r="M32" s="40"/>
+      <x:c r="N32" s="40"/>
+      <x:c r="O32" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.04 Fishing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B33" s="40" t="n"/>
-      <x:c r="C33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D33" s="40" t="n"/>
-      <x:c r="E33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DETACHED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F33" s="40" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Detached comparison boundary for LEAP All demand aggregated/Other sector. Sums agriculture, fishing, non-specified others, and non-energy use without making flow 17 a child of flow 16 or changing the detailed LEAP structure.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MIXED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03 Agriculture; 16.04 Fishing; 16.05 Non-specified others; 17 Non-energy use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">other_sector_comparison</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">all_demand_aggregated_esto_rollup_rules</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M33" s="40" t="n"/>
-      <x:c r="N33" s="40" t="n"/>
-      <x:c r="O33" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A33" s="40" t="str">
+        <x:v>16.04 Fishing</x:v>
+      </x:c>
+      <x:c r="B33" s="40"/>
+      <x:c r="C33" s="40" t="str">
+        <x:v>16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="D33" s="40"/>
+      <x:c r="E33" s="40" t="str">
+        <x:v>DETACHED</x:v>
+      </x:c>
+      <x:c r="F33" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G33" s="40" t="str">
+        <x:v>Disabled after the global clean-slate cutover: Non-energy use is mapped as its own flow 17 branch, so the former combined Other-sector subtotal must not be generated.</x:v>
+      </x:c>
+      <x:c r="H33" s="40" t="str">
+        <x:v>MIXED</x:v>
+      </x:c>
+      <x:c r="I33" s="40" t="str">
+        <x:v>16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="J33" s="40" t="str">
+        <x:v>16.03 Agriculture; 16.04 Fishing; 16.05 Non-specified others; 17 Non-energy use</x:v>
+      </x:c>
+      <x:c r="K33" s="40" t="str">
+        <x:v>other_sector_comparison</x:v>
+      </x:c>
+      <x:c r="L33" s="40" t="str">
+        <x:v>all_demand_aggregated_esto_rollup_rules</x:v>
+      </x:c>
+      <x:c r="M33" s="40"/>
+      <x:c r="N33" s="40"/>
+      <x:c r="O33" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.05 Non-specified others</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B34" s="40" t="n"/>
-      <x:c r="C34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D34" s="40" t="n"/>
-      <x:c r="E34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DETACHED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F34" s="40" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Detached comparison boundary for LEAP All demand aggregated/Other sector. Sums agriculture, fishing, non-specified others, and non-energy use without making flow 17 a child of flow 16 or changing the detailed LEAP structure.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MIXED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03 Agriculture; 16.04 Fishing; 16.05 Non-specified others; 17 Non-energy use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">other_sector_comparison</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">all_demand_aggregated_esto_rollup_rules</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M34" s="40" t="n"/>
-      <x:c r="N34" s="40" t="n"/>
-      <x:c r="O34" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A34" s="40" t="str">
+        <x:v>16.05 Non-specified others</x:v>
+      </x:c>
+      <x:c r="B34" s="40"/>
+      <x:c r="C34" s="40" t="str">
+        <x:v>16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="D34" s="40"/>
+      <x:c r="E34" s="40" t="str">
+        <x:v>DETACHED</x:v>
+      </x:c>
+      <x:c r="F34" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G34" s="40" t="str">
+        <x:v>Disabled after the global clean-slate cutover: Non-energy use is mapped as its own flow 17 branch, so the former combined Other-sector subtotal must not be generated.</x:v>
+      </x:c>
+      <x:c r="H34" s="40" t="str">
+        <x:v>MIXED</x:v>
+      </x:c>
+      <x:c r="I34" s="40" t="str">
+        <x:v>16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="J34" s="40" t="str">
+        <x:v>16.03 Agriculture; 16.04 Fishing; 16.05 Non-specified others; 17 Non-energy use</x:v>
+      </x:c>
+      <x:c r="K34" s="40" t="str">
+        <x:v>other_sector_comparison</x:v>
+      </x:c>
+      <x:c r="L34" s="40" t="str">
+        <x:v>all_demand_aggregated_esto_rollup_rules</x:v>
+      </x:c>
+      <x:c r="M34" s="40"/>
+      <x:c r="N34" s="40"/>
+      <x:c r="O34" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17 Non-energy use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B35" s="40" t="n"/>
-      <x:c r="C35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D35" s="40" t="n"/>
-      <x:c r="E35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DETACHED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F35" s="40" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Detached comparison boundary for LEAP All demand aggregated/Other sector. Sums agriculture, fishing, non-specified others, and non-energy use without making flow 17 a child of flow 16 or changing the detailed LEAP structure.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MIXED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03 Agriculture; 16.04 Fishing; 16.05 Non-specified others; 17 Non-energy use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">other_sector_comparison</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">all_demand_aggregated_esto_rollup_rules</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M35" s="40" t="n"/>
-      <x:c r="N35" s="40" t="n"/>
-      <x:c r="O35" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A35" s="40" t="str">
+        <x:v>17 Non-energy use</x:v>
+      </x:c>
+      <x:c r="B35" s="40"/>
+      <x:c r="C35" s="40" t="str">
+        <x:v>16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="D35" s="40"/>
+      <x:c r="E35" s="40" t="str">
+        <x:v>DETACHED</x:v>
+      </x:c>
+      <x:c r="F35" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G35" s="40" t="str">
+        <x:v>Disabled after the global clean-slate cutover: Non-energy use is mapped as its own flow 17 branch, so the former combined Other-sector subtotal must not be generated.</x:v>
+      </x:c>
+      <x:c r="H35" s="40" t="str">
+        <x:v>MIXED</x:v>
+      </x:c>
+      <x:c r="I35" s="40" t="str">
+        <x:v>16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="J35" s="40" t="str">
+        <x:v>16.03 Agriculture; 16.04 Fishing; 16.05 Non-specified others; 17 Non-energy use</x:v>
+      </x:c>
+      <x:c r="K35" s="40" t="str">
+        <x:v>other_sector_comparison</x:v>
+      </x:c>
+      <x:c r="L35" s="40" t="str">
+        <x:v>all_demand_aggregated_esto_rollup_rules</x:v>
+      </x:c>
+      <x:c r="M35" s="40"/>
+      <x:c r="N35" s="40"/>
+      <x:c r="O35" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -29519,166 +29472,112 @@
       <x:c r="N25" s="40" t="n"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02_agriculture_and_fishing</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B26" s="40" t="n"/>
-      <x:c r="C26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D26" s="40" t="n"/>
-      <x:c r="E26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DETACHED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F26" s="40" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Detached comparison boundary matching LEAP All demand aggregated/Other sector. Sums agriculture and fishing, non-specified others, and non-energy use while retaining the ordinary NINTH sector hierarchy.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MIXED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02_agriculture_and_fishing; 16_05_nonspecified_others; 17_nonenergy_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">other_sector_comparison</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L26" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">all_demand_aggregated_ninth_rollup_rules</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M26" s="40" t="n"/>
-      <x:c r="N26" s="40" t="n"/>
+      <x:c r="A26" s="40" t="str">
+        <x:v>16_02_agriculture_and_fishing</x:v>
+      </x:c>
+      <x:c r="B26" s="40"/>
+      <x:c r="C26" s="40" t="str">
+        <x:v>16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="D26" s="40"/>
+      <x:c r="E26" s="40" t="str">
+        <x:v>DETACHED</x:v>
+      </x:c>
+      <x:c r="F26" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G26" s="40" t="str">
+        <x:v>Disabled after the global clean-slate cutover: Non-energy use is mapped as its own flow 17 branch, so the former combined Other-sector subtotal must not be generated.</x:v>
+      </x:c>
+      <x:c r="H26" s="40" t="str">
+        <x:v>MIXED</x:v>
+      </x:c>
+      <x:c r="I26" s="40" t="str">
+        <x:v>16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="J26" s="40" t="str">
+        <x:v>16_02_agriculture_and_fishing; 16_05_nonspecified_others; 17_nonenergy_use</x:v>
+      </x:c>
+      <x:c r="K26" s="40" t="str">
+        <x:v>other_sector_comparison</x:v>
+      </x:c>
+      <x:c r="L26" s="40" t="str">
+        <x:v>all_demand_aggregated_ninth_rollup_rules</x:v>
+      </x:c>
+      <x:c r="M26" s="40"/>
+      <x:c r="N26" s="40"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_05_nonspecified_others</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B27" s="40" t="n"/>
-      <x:c r="C27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D27" s="40" t="n"/>
-      <x:c r="E27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DETACHED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F27" s="40" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Detached comparison boundary matching LEAP All demand aggregated/Other sector. Sums agriculture and fishing, non-specified others, and non-energy use while retaining the ordinary NINTH sector hierarchy.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MIXED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02_agriculture_and_fishing; 16_05_nonspecified_others; 17_nonenergy_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">other_sector_comparison</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L27" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">all_demand_aggregated_ninth_rollup_rules</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M27" s="40" t="n"/>
-      <x:c r="N27" s="40" t="n"/>
+      <x:c r="A27" s="40" t="str">
+        <x:v>16_05_nonspecified_others</x:v>
+      </x:c>
+      <x:c r="B27" s="40"/>
+      <x:c r="C27" s="40" t="str">
+        <x:v>16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="D27" s="40"/>
+      <x:c r="E27" s="40" t="str">
+        <x:v>DETACHED</x:v>
+      </x:c>
+      <x:c r="F27" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G27" s="40" t="str">
+        <x:v>Disabled after the global clean-slate cutover: Non-energy use is mapped as its own flow 17 branch, so the former combined Other-sector subtotal must not be generated.</x:v>
+      </x:c>
+      <x:c r="H27" s="40" t="str">
+        <x:v>MIXED</x:v>
+      </x:c>
+      <x:c r="I27" s="40" t="str">
+        <x:v>16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="J27" s="40" t="str">
+        <x:v>16_02_agriculture_and_fishing; 16_05_nonspecified_others; 17_nonenergy_use</x:v>
+      </x:c>
+      <x:c r="K27" s="40" t="str">
+        <x:v>other_sector_comparison</x:v>
+      </x:c>
+      <x:c r="L27" s="40" t="str">
+        <x:v>all_demand_aggregated_ninth_rollup_rules</x:v>
+      </x:c>
+      <x:c r="M27" s="40"/>
+      <x:c r="N27" s="40"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17_nonenergy_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B28" s="40" t="n"/>
-      <x:c r="C28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D28" s="40" t="n"/>
-      <x:c r="E28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DETACHED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F28" s="40" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Detached comparison boundary matching LEAP All demand aggregated/Other sector. Sums agriculture and fishing, non-specified others, and non-energy use while retaining the ordinary NINTH sector hierarchy.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MIXED</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16_02_agriculture_and_fishing; 16_05_nonspecified_others; 17_nonenergy_use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">other_sector_comparison</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L28" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">all_demand_aggregated_ninth_rollup_rules</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M28" s="40" t="n"/>
-      <x:c r="N28" s="40" t="n"/>
+      <x:c r="A28" s="40" t="str">
+        <x:v>17_nonenergy_use</x:v>
+      </x:c>
+      <x:c r="B28" s="40"/>
+      <x:c r="C28" s="40" t="str">
+        <x:v>16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="D28" s="40"/>
+      <x:c r="E28" s="40" t="str">
+        <x:v>DETACHED</x:v>
+      </x:c>
+      <x:c r="F28" s="44" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G28" s="40" t="str">
+        <x:v>Disabled after the global clean-slate cutover: Non-energy use is mapped as its own flow 17 branch, so the former combined Other-sector subtotal must not be generated.</x:v>
+      </x:c>
+      <x:c r="H28" s="40" t="str">
+        <x:v>MIXED</x:v>
+      </x:c>
+      <x:c r="I28" s="40" t="str">
+        <x:v>16_02-16_05,17 Other sector including non-energy (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="J28" s="40" t="str">
+        <x:v>16_02_agriculture_and_fishing; 16_05_nonspecified_others; 17_nonenergy_use</x:v>
+      </x:c>
+      <x:c r="K28" s="40" t="str">
+        <x:v>other_sector_comparison</x:v>
+      </x:c>
+      <x:c r="L28" s="40" t="str">
+        <x:v>all_demand_aggregated_ninth_rollup_rules</x:v>
+      </x:c>
+      <x:c r="M28" s="40"/>
+      <x:c r="N28" s="40"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="40" t="inlineStr">
@@ -31467,20 +31366,14 @@
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">All demand aggregated/Other sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C6" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A6" s="40" t="str">
+        <x:v>All demand aggregated/Other sector</x:v>
+      </x:c>
+      <x:c r="B6" s="40" t="str">
+        <x:v>16.03-16.05 Other sector (all demand aggregate)</x:v>
+      </x:c>
+      <x:c r="C6" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -33082,20 +32975,14 @@
       </x:c>
     </x:row>
     <x:row r="101">
-      <x:c r="A101" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Other sector</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B101" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16.03-16.05,17 Other sector including non-energy (all demand aggregate)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C101" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BOTH</x:t>
-        </x:is>
+      <x:c r="A101" s="40" t="str">
+        <x:v>Other sector</x:v>
+      </x:c>
+      <x:c r="B101" s="40" t="str">
+        <x:v>16.03-16.05 Other sector</x:v>
+      </x:c>
+      <x:c r="C101" s="40" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -33995,6 +33882,17 @@
         <x:is>
           <x:t xml:space="preserve">BOTH</x:t>
         </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>All demand aggregated/Non Energy Use</x:v>
+      </x:c>
+      <x:c r="B155" t="str">
+        <x:v>17 Non-energy use</x:v>
+      </x:c>
+      <x:c r="C155" t="str">
+        <x:v>BOTH</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -36861,6 +36759,14 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>All demand aggregated/Non Energy Use</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>17_nonenergy_use</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
codex: finalize LNG inclusive mapping artifacts
Verification: 18 focused LNG, anchor-resume, Stage 3 dependency, and anchor dtype tests passed.
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R58f9e8ceb4e745d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="Raf8807a78d944ca7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R1d5a0fff862b4d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="Rdf11deb6e4fb4293"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="R0d038d1cd52b48ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="Rc9979826f4e94142"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Ref05696c52b44ffb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="R91f95748ff464e8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="R4e1db5856d2a492d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="R6b0a7a7f876b405b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R6ff27d27ec104476"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="Rceb8e2bc7aca47e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="R40f79ecfef7446e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="Rf08593aa8f0e49a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R7c9381d627594087"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="R9f8f854328184e97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4edb98795465493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_esto" sheetId="2" r:id="R3b0fa37178854cf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_esto" sheetId="3" r:id="R53df47164bdc4bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_sector_to_ninth" sheetId="4" r:id="R7602f986d5a042f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_fuel_to_ninth" sheetId="5" r:id="Rc331932701624b18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_sector_to_esto" sheetId="6" r:id="R32d187ea3e9f43ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_fuel_to_esto" sheetId="7" r:id="Rb67eb36588c04189"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_leap_key_pairs" sheetId="8" r:id="R4f76b452b748462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_key_pairs" sheetId="9" r:id="Rf4798a92c184479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_esto_extended_pairs" sheetId="10" r:id="Rdcdb5178e9954398"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extra_ninth_key_pairs" sheetId="11" r:id="R73abb770921a4670"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exceptions" sheetId="12" r:id="Rc74ef1af249a4724"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leap_rollup_rules" sheetId="13" r:id="Rbc7bbdc65d094421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="esto_rollup_rules" sheetId="14" r:id="R4534d6d87eec4164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ninth_rollup_rules" sheetId="15" r:id="R39e6a58bf682486d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rollup_label_overrides" sheetId="16" r:id="R0b980d0c43fe4524"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -350,13 +350,13 @@
     <xdr:ext cx="11239500" cy="2238375"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="/xl/media/image1.png"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8366742129df481b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbb75903a49154c8c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1019,7 +1019,7 @@
     <x:mergeCell ref="A4:H4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd09e29719ef44816"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re699eb7f25544fae"/>
 </x:worksheet>
 </file>
 
@@ -23970,10 +23970,8 @@
         </x:is>
       </x:c>
       <x:c r="B2" s="43" t="n"/>
-      <x:c r="C2" s="43" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gas processing plants</x:t>
-        </x:is>
+      <x:c r="C2" s="43" t="str">
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="D2" s="43" t="n"/>
       <x:c r="E2" s="43" t="inlineStr">
@@ -24017,10 +24015,8 @@
         </x:is>
       </x:c>
       <x:c r="B3" s="44" t="n"/>
-      <x:c r="C3" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gas processing plants</x:t>
-        </x:is>
+      <x:c r="C3" s="44" t="str">
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="D3" s="44" t="n"/>
       <x:c r="E3" s="44" t="inlineStr">
@@ -24064,10 +24060,8 @@
         </x:is>
       </x:c>
       <x:c r="B4" s="44" t="n"/>
-      <x:c r="C4" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gas processing plants</x:t>
-        </x:is>
+      <x:c r="C4" s="44" t="str">
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="D4" s="44" t="n"/>
       <x:c r="E4" s="44" t="inlineStr">
@@ -24111,10 +24105,8 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="44" t="n"/>
-      <x:c r="C5" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gas processing plants</x:t>
-        </x:is>
+      <x:c r="C5" s="44" t="str">
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="D5" s="44" t="n"/>
       <x:c r="E5" s="44" t="inlineStr">
@@ -24158,10 +24150,8 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="44" t="n"/>
-      <x:c r="C6" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gas processing plants</x:t>
-        </x:is>
+      <x:c r="C6" s="44" t="str">
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="D6" s="44" t="n"/>
       <x:c r="E6" s="44" t="inlineStr">
@@ -24569,10 +24559,8 @@
         </x:is>
       </x:c>
       <x:c r="B15" s="44" t="n"/>
-      <x:c r="C15" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Liquefaction/regasification plants</x:t>
-        </x:is>
+      <x:c r="C15" s="44" t="str">
+        <x:v>Liquefaction/regasification plants (including own use)</x:v>
       </x:c>
       <x:c r="D15" s="44" t="n"/>
       <x:c r="E15" s="44" t="inlineStr">
@@ -24591,10 +24579,8 @@
       <x:c r="H15" s="44" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I15" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gas processing plants</x:t>
-        </x:is>
+      <x:c r="I15" s="44" t="str">
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="J15" s="44" t="inlineStr">
         <x:is>
@@ -24616,10 +24602,8 @@
         </x:is>
       </x:c>
       <x:c r="B16" s="44" t="n"/>
-      <x:c r="C16" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Liquefaction/regasification plants</x:t>
-        </x:is>
+      <x:c r="C16" s="44" t="str">
+        <x:v>Liquefaction/regasification plants (including own use)</x:v>
       </x:c>
       <x:c r="D16" s="44" t="n"/>
       <x:c r="E16" s="44" t="inlineStr">
@@ -24638,10 +24622,8 @@
       <x:c r="H16" s="44" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I16" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gas processing plants</x:t>
-        </x:is>
+      <x:c r="I16" s="44" t="str">
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="J16" s="44" t="inlineStr">
         <x:is>
@@ -27784,7 +27766,7 @@
       </x:c>
       <x:c r="B86" t="str"/>
       <x:c r="C86" t="str">
-        <x:v>Liquefaction/regasification plants</x:v>
+        <x:v>Liquefaction/regasification plants (including own use)</x:v>
       </x:c>
       <x:c r="D86" t="str"/>
       <x:c r="E86" t="str">
@@ -27800,7 +27782,7 @@
         <x:v>TRUE</x:v>
       </x:c>
       <x:c r="I86" t="str">
-        <x:v>Gas processing plants</x:v>
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="J86" t="str">
         <x:v>LNG regasification; NG Liquefaction</x:v>
@@ -27819,7 +27801,7 @@
       </x:c>
       <x:c r="B87" t="str"/>
       <x:c r="C87" t="str">
-        <x:v>Gas processing plants</x:v>
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="D87" t="str"/>
       <x:c r="E87" t="str">
@@ -39402,15 +39384,11 @@
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gas processing plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B49" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.06 Gas processing plants</x:t>
-        </x:is>
+      <x:c r="A49" s="44" t="str">
+        <x:v>Gas processing plants (including own use)</x:v>
+      </x:c>
+      <x:c r="B49" s="44" t="str">
+        <x:v>09.06 Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="C49" s="44" t="inlineStr">
         <x:is>
@@ -40065,15 +40043,11 @@
       </x:c>
     </x:row>
     <x:row r="88">
-      <x:c r="A88" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Liquefaction/regasification plants</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B88" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">09.06.02 Liquefaction/regasification plants</x:t>
-        </x:is>
+      <x:c r="A88" s="44" t="str">
+        <x:v>Liquefaction/regasification plants (including own use)</x:v>
+      </x:c>
+      <x:c r="B88" s="44" t="str">
+        <x:v>09.06.02 Liquefaction/regasification plants (including own use)</x:v>
       </x:c>
       <x:c r="C88" s="44" t="inlineStr">
         <x:is>
@@ -42921,10 +42895,8 @@
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gas processing plants</x:t>
-        </x:is>
+      <x:c r="A39" s="44" t="str">
+        <x:v>Gas processing plants (including own use)</x:v>
       </x:c>
       <x:c r="B39" s="44" t="inlineStr">
         <x:is>
@@ -43209,10 +43181,8 @@
       </x:c>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="44" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Liquefaction/regasification plants</x:t>
-        </x:is>
+      <x:c r="A63" s="44" t="str">
+        <x:v>Liquefaction/regasification plants (including own use)</x:v>
       </x:c>
       <x:c r="B63" s="44" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
codex: promote electrolyser green electricity mapping
Refresh the generated pair authority and compatibility master after accepting the Green electricity target pair. Verified all three generated mapping directions.
</commit_message>
<xml_diff>
--- a/config/outlook_mappings_single_axis.xlsx
+++ b/config/outlook_mappings_single_axis.xlsx
@@ -53195,7 +53195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B968"/>
+  <dimension ref="A1:B969"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="47" min="1" max="1"/>
@@ -64818,6 +64818,18 @@
         </is>
       </c>
     </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>09.13.01 Electrolysers</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>20 Green electricity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>